<commit_message>
site build 2026-10-08 16:50
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB21"/>
+  <dimension ref="A1:AB22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -943,7 +943,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -953,38 +953,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>B-</t>
+          <t>CCC-</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="I9" t="n">
-        <v>14</v>
-      </c>
-      <c r="J9" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="L9" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" t="n">
-        <v>5.2</v>
+          <t>None (technical surveillance only)</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>70</v>
+      </c>
+      <c r="U9" t="n">
+        <v>17.5</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -993,31 +979,31 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>reports/ghana-sovereign-credit.md</t>
+          <t>reports/gabon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
       <c r="E10" t="inlineStr">
         <is>
           <t>Caa1</t>
@@ -1025,20 +1011,23 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>None (Article IV / Post-Financing Assessment)</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
-        <v>-6.8</v>
+          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I10" t="n">
+        <v>14</v>
+      </c>
+      <c r="J10" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="L10" t="n">
-        <v>80.59999999999999</v>
+        <v>12</v>
       </c>
       <c r="M10" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="X10" t="n">
-        <v>0.506</v>
+        <v>5.2</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1047,14 +1036,14 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>reports/iraq-sovereign-credit.md</t>
+          <t>reports/ghana-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1064,44 +1053,35 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>EFF (4-year) + RSF</t>
-        </is>
-      </c>
-      <c r="I11" t="n">
-        <v>6</v>
+          <t>None (Article IV / Post-Financing Assessment)</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>-6.8</v>
       </c>
       <c r="L11" t="n">
-        <v>28.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M11" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="P11" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="R11" t="n">
-        <v>-2.8</v>
+        <v>9.6</v>
       </c>
       <c r="X11" t="n">
-        <v>3.95</v>
+        <v>0.506</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1110,61 +1090,61 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>reports/jordan-sovereign-credit.md</t>
+          <t>reports/iraq-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year) + RSF</t>
+        </is>
       </c>
       <c r="I12" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="J12" t="n">
-        <v>1.95</v>
+        <v>6</v>
       </c>
       <c r="L12" t="n">
-        <v>14.702</v>
+        <v>28.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="P12" t="n">
-        <v>68.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q12" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="S12" t="n">
-        <v>33</v>
+        <v>-5.2</v>
+      </c>
+      <c r="R12" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="X12" t="n">
+        <v>3.95</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -1173,58 +1153,61 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>reports/kenya-sovereign-credit.md</t>
+          <t>reports/jordan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ba1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>FCL (2-year, precautionary)</t>
-        </is>
+          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>6.8</v>
       </c>
       <c r="I13" t="n">
-        <v>2.25</v>
+        <v>8.75</v>
+      </c>
+      <c r="J13" t="n">
+        <v>1.95</v>
       </c>
       <c r="L13" t="n">
-        <v>55.65</v>
-      </c>
-      <c r="M13" t="n">
-        <v>5.5</v>
+        <v>14.702</v>
       </c>
       <c r="P13" t="n">
-        <v>66.5</v>
+        <v>68.5</v>
       </c>
       <c r="Q13" t="n">
-        <v>-3</v>
+        <v>-6.4</v>
       </c>
       <c r="S13" t="n">
-        <v>11.5</v>
+        <v>33</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -1233,58 +1216,58 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>reports/morocco-sovereign-credit.md</t>
+          <t>reports/kenya-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba1</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>15.39</v>
+          <t>FCL (2-year, precautionary)</t>
+        </is>
       </c>
       <c r="I14" t="n">
-        <v>23</v>
-      </c>
-      <c r="J14" t="n">
-        <v>7.61</v>
+        <v>2.25</v>
       </c>
       <c r="L14" t="n">
-        <v>54.98</v>
+        <v>55.65</v>
+      </c>
+      <c r="M14" t="n">
+        <v>5.5</v>
       </c>
       <c r="P14" t="n">
-        <v>32.3</v>
+        <v>66.5</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>-3</v>
       </c>
       <c r="S14" t="n">
-        <v>55</v>
+        <v>11.5</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -1293,34 +1276,34 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>reports/nigeria-sovereign-credit.md</t>
+          <t>reports/morocco-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Baa3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -1328,20 +1311,23 @@
           <t>None (Article IV)</t>
         </is>
       </c>
-      <c r="G15" t="n">
-        <v>2.1</v>
+      <c r="H15" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="I15" t="n">
+        <v>23</v>
+      </c>
+      <c r="J15" t="n">
+        <v>7.61</v>
       </c>
       <c r="L15" t="n">
-        <v>18.38</v>
-      </c>
-      <c r="M15" t="n">
-        <v>5</v>
+        <v>54.98</v>
       </c>
       <c r="P15" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>0.65</v>
+        <v>32.3</v>
+      </c>
+      <c r="S15" t="n">
+        <v>55</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -1350,47 +1336,55 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>reports/oman-sovereign-credit.md</t>
+          <t>reports/nigeria-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>Baa3</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I16" t="n">
-        <v>3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>1.8</v>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="M16" t="n">
+        <v>5</v>
       </c>
       <c r="P16" t="n">
-        <v>132</v>
+        <v>34.7</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>0.65</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -1399,58 +1393,47 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/oman-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Europe</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing)</t>
-        </is>
-      </c>
-      <c r="G17" t="n">
-        <v>3.3</v>
+          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
+        </is>
       </c>
       <c r="H17" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I17" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J17" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="K17" t="n">
-        <v>-4.1</v>
+        <v>1.8</v>
       </c>
       <c r="P17" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -1459,29 +1442,29 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1491,29 +1474,26 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
+          <t>PCI (36-month, non-financing)</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>3.3</v>
       </c>
       <c r="H18" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I18" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J18" t="n">
-        <v>2.85</v>
+        <v>3.55</v>
       </c>
       <c r="K18" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="L18" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="M18" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="Q18" t="n">
-        <v>-4.5</v>
+        <v>-4.1</v>
+      </c>
+      <c r="P18" t="n">
+        <v>43.3</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -1522,34 +1502,34 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1558,31 +1538,25 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>29.73</v>
+        <v>4.4</v>
       </c>
       <c r="I19" t="n">
-        <v>37</v>
+        <v>7.25</v>
       </c>
       <c r="J19" t="n">
-        <v>7.27</v>
+        <v>2.85</v>
       </c>
       <c r="K19" t="n">
-        <v>-2.7</v>
+        <v>-1.6</v>
       </c>
       <c r="L19" t="n">
-        <v>61.56</v>
-      </c>
-      <c r="N19" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="O19" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="P19" t="n">
-        <v>29.5</v>
+        <v>63.5</v>
+      </c>
+      <c r="M19" t="n">
+        <v>5.8</v>
       </c>
       <c r="Q19" t="n">
-        <v>-5.2</v>
+        <v>-4.5</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -1591,14 +1565,14 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1608,41 +1582,50 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>EFF (4-year)</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I20" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J20" t="n">
-        <v>7.9</v>
+        <v>7.27</v>
+      </c>
+      <c r="K20" t="n">
+        <v>-2.7</v>
       </c>
       <c r="L20" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="M20" t="n">
-        <v>5.6</v>
+        <v>61.56</v>
+      </c>
+      <c r="N20" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O20" t="n">
+        <v>31.8</v>
       </c>
       <c r="P20" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>-5.2</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -1651,71 +1634,131 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>EFF (4-year)</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>16</v>
+      </c>
+      <c r="J21" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L21" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="M21" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="P21" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB21" t="inlineStr">
+        <is>
+          <t>reports/ukraine-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
           <t>Uzbekistan</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>CIS</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D22" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>Ba2</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>None (Article IV)</t>
         </is>
       </c>
-      <c r="G21" t="n">
+      <c r="G22" t="n">
         <v>6.8</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H22" t="n">
         <v>6.2</v>
       </c>
-      <c r="I21" t="n">
+      <c r="I22" t="n">
         <v>14</v>
       </c>
-      <c r="J21" t="n">
+      <c r="J22" t="n">
         <v>7.8</v>
       </c>
-      <c r="L21" t="n">
+      <c r="L22" t="n">
         <v>72.13</v>
       </c>
-      <c r="M21" t="n">
+      <c r="M22" t="n">
         <v>12</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P22" t="n">
         <v>27</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q22" t="n">
         <v>-2.1</v>
       </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="AB21" t="inlineStr">
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
         <is>
           <t>reports/uzbekistan-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-08 17:15
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB22"/>
+  <dimension ref="A1:AB23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -820,7 +820,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -830,41 +830,38 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>EFF/ECF ($3.5B) and RSF ($1.3B) completed Jun-26</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>6</v>
+          <t>Post-Financing Assessment (PFA); ECF/EFF/RSF completed Jul-25</t>
+        </is>
       </c>
       <c r="H7" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I7" t="n">
-        <v>3</v>
-      </c>
-      <c r="J7" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="O7" t="n">
+        <v>30</v>
       </c>
       <c r="P7" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>-3.8</v>
+        <v>43</v>
+      </c>
+      <c r="S7" t="n">
+        <v>20</v>
+      </c>
+      <c r="T7" t="n">
+        <v>12</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -873,61 +870,58 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>reports/cote-d-ivoire-sovereign-credit.md</t>
+          <t>reports/cameroon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Cote d'Ivoire</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EFF</t>
-        </is>
+          <t>EFF/ECF ($3.5B) and RSF ($1.3B) completed Jun-26</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>6</v>
       </c>
       <c r="H8" t="n">
-        <v>12.7</v>
+        <v>1.2</v>
       </c>
       <c r="I8" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="J8" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="M8" t="n">
-        <v>7.5</v>
+        <v>1.8</v>
       </c>
       <c r="P8" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="R8" t="n">
-        <v>4</v>
-      </c>
-      <c r="S8" t="n">
-        <v>50</v>
+        <v>55.1</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>-3.8</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -936,41 +930,61 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>reports/egypt-sovereign-credit.md</t>
+          <t>reports/cote-d-ivoire-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Gabon</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>CCC-</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>None (technical surveillance only)</t>
-        </is>
+          <t>EFF</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="I9" t="n">
+        <v>19</v>
+      </c>
+      <c r="J9" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="M9" t="n">
+        <v>7.5</v>
       </c>
       <c r="P9" t="n">
-        <v>70</v>
-      </c>
-      <c r="U9" t="n">
-        <v>17.5</v>
+        <v>79.7</v>
+      </c>
+      <c r="R9" t="n">
+        <v>4</v>
+      </c>
+      <c r="S9" t="n">
+        <v>50</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -979,14 +993,14 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>reports/gabon-sovereign-credit.md</t>
+          <t>reports/egypt-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -996,38 +1010,24 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>B-</t>
+          <t>CCC-</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="I10" t="n">
-        <v>14</v>
-      </c>
-      <c r="J10" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="L10" t="n">
-        <v>12</v>
-      </c>
-      <c r="M10" t="n">
-        <v>5.2</v>
+          <t>None (technical surveillance only)</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>70</v>
+      </c>
+      <c r="U10" t="n">
+        <v>17.5</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1036,31 +1036,31 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>reports/ghana-sovereign-credit.md</t>
+          <t>reports/gabon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
       <c r="E11" t="inlineStr">
         <is>
           <t>Caa1</t>
@@ -1068,20 +1068,23 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>None (Article IV / Post-Financing Assessment)</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
-        <v>-6.8</v>
+          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I11" t="n">
+        <v>14</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="L11" t="n">
-        <v>80.59999999999999</v>
+        <v>12</v>
       </c>
       <c r="M11" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="X11" t="n">
-        <v>0.506</v>
+        <v>5.2</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1090,14 +1093,14 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>reports/iraq-sovereign-credit.md</t>
+          <t>reports/ghana-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1107,44 +1110,35 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>EFF (4-year) + RSF</t>
-        </is>
-      </c>
-      <c r="I12" t="n">
-        <v>6</v>
+          <t>None (Article IV / Post-Financing Assessment)</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>-6.8</v>
       </c>
       <c r="L12" t="n">
-        <v>28.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M12" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="P12" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="R12" t="n">
-        <v>-2.8</v>
+        <v>9.6</v>
       </c>
       <c r="X12" t="n">
-        <v>3.95</v>
+        <v>0.506</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -1153,61 +1147,61 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>reports/jordan-sovereign-credit.md</t>
+          <t>reports/iraq-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year) + RSF</t>
+        </is>
       </c>
       <c r="I13" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1.95</v>
+        <v>6</v>
       </c>
       <c r="L13" t="n">
-        <v>14.702</v>
+        <v>28.5</v>
+      </c>
+      <c r="M13" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="P13" t="n">
-        <v>68.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q13" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="S13" t="n">
-        <v>33</v>
+        <v>-5.2</v>
+      </c>
+      <c r="R13" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="X13" t="n">
+        <v>3.95</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -1216,58 +1210,61 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>reports/kenya-sovereign-credit.md</t>
+          <t>reports/jordan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Ba1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>FCL (2-year, precautionary)</t>
-        </is>
+          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>6.8</v>
       </c>
       <c r="I14" t="n">
-        <v>2.25</v>
+        <v>8.75</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1.95</v>
       </c>
       <c r="L14" t="n">
-        <v>55.65</v>
-      </c>
-      <c r="M14" t="n">
-        <v>5.5</v>
+        <v>14.702</v>
       </c>
       <c r="P14" t="n">
-        <v>66.5</v>
+        <v>68.5</v>
       </c>
       <c r="Q14" t="n">
-        <v>-3</v>
+        <v>-6.4</v>
       </c>
       <c r="S14" t="n">
-        <v>11.5</v>
+        <v>33</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -1276,58 +1273,58 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>reports/morocco-sovereign-credit.md</t>
+          <t>reports/kenya-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>15.39</v>
+          <t>FCL (2-year, precautionary)</t>
+        </is>
       </c>
       <c r="I15" t="n">
-        <v>23</v>
-      </c>
-      <c r="J15" t="n">
-        <v>7.61</v>
+        <v>2.25</v>
       </c>
       <c r="L15" t="n">
-        <v>54.98</v>
+        <v>55.65</v>
+      </c>
+      <c r="M15" t="n">
+        <v>5.5</v>
       </c>
       <c r="P15" t="n">
-        <v>32.3</v>
+        <v>66.5</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>-3</v>
       </c>
       <c r="S15" t="n">
-        <v>55</v>
+        <v>11.5</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -1336,34 +1333,34 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>reports/nigeria-sovereign-credit.md</t>
+          <t>reports/morocco-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Baa3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1371,20 +1368,23 @@
           <t>None (Article IV)</t>
         </is>
       </c>
-      <c r="G16" t="n">
-        <v>2.1</v>
+      <c r="H16" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="I16" t="n">
+        <v>23</v>
+      </c>
+      <c r="J16" t="n">
+        <v>7.61</v>
       </c>
       <c r="L16" t="n">
-        <v>18.38</v>
-      </c>
-      <c r="M16" t="n">
-        <v>5</v>
+        <v>54.98</v>
       </c>
       <c r="P16" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Q16" t="n">
-        <v>0.65</v>
+        <v>32.3</v>
+      </c>
+      <c r="S16" t="n">
+        <v>55</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -1393,47 +1393,55 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>reports/oman-sovereign-credit.md</t>
+          <t>reports/nigeria-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>Baa3</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I17" t="n">
-        <v>3</v>
-      </c>
-      <c r="J17" t="n">
-        <v>1.8</v>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L17" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="M17" t="n">
+        <v>5</v>
       </c>
       <c r="P17" t="n">
-        <v>132</v>
+        <v>34.7</v>
+      </c>
+      <c r="Q17" t="n">
+        <v>0.65</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -1442,58 +1450,47 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/oman-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Europe</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing)</t>
-        </is>
-      </c>
-      <c r="G18" t="n">
-        <v>3.3</v>
+          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
+        </is>
       </c>
       <c r="H18" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I18" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J18" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="K18" t="n">
-        <v>-4.1</v>
+        <v>1.8</v>
       </c>
       <c r="P18" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -1502,29 +1499,29 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -1534,29 +1531,26 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
+          <t>PCI (36-month, non-financing)</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>3.3</v>
       </c>
       <c r="H19" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I19" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J19" t="n">
-        <v>2.85</v>
+        <v>3.55</v>
       </c>
       <c r="K19" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="L19" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="M19" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="Q19" t="n">
-        <v>-4.5</v>
+        <v>-4.1</v>
+      </c>
+      <c r="P19" t="n">
+        <v>43.3</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -1565,34 +1559,34 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -1601,31 +1595,25 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>29.73</v>
+        <v>4.4</v>
       </c>
       <c r="I20" t="n">
-        <v>37</v>
+        <v>7.25</v>
       </c>
       <c r="J20" t="n">
-        <v>7.27</v>
+        <v>2.85</v>
       </c>
       <c r="K20" t="n">
-        <v>-2.7</v>
+        <v>-1.6</v>
       </c>
       <c r="L20" t="n">
-        <v>61.56</v>
-      </c>
-      <c r="N20" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="O20" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="P20" t="n">
-        <v>29.5</v>
+        <v>63.5</v>
+      </c>
+      <c r="M20" t="n">
+        <v>5.8</v>
       </c>
       <c r="Q20" t="n">
-        <v>-5.2</v>
+        <v>-4.5</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -1634,14 +1622,14 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1651,41 +1639,50 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>EFF (4-year)</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I21" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J21" t="n">
-        <v>7.9</v>
+        <v>7.27</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-2.7</v>
       </c>
       <c r="L21" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="M21" t="n">
-        <v>5.6</v>
+        <v>61.56</v>
+      </c>
+      <c r="N21" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O21" t="n">
+        <v>31.8</v>
       </c>
       <c r="P21" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>-5.2</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -1694,71 +1691,131 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>EFF (4-year)</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="I22" t="n">
+        <v>16</v>
+      </c>
+      <c r="J22" t="n">
+        <v>7.9</v>
+      </c>
+      <c r="L22" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="M22" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="P22" t="n">
+        <v>98.40000000000001</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB22" t="inlineStr">
+        <is>
+          <t>reports/ukraine-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>Uzbekistan</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>CIS</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>BB</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Ba2</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>None (Article IV)</t>
         </is>
       </c>
-      <c r="G22" t="n">
+      <c r="G23" t="n">
         <v>6.8</v>
       </c>
-      <c r="H22" t="n">
+      <c r="H23" t="n">
         <v>6.2</v>
       </c>
-      <c r="I22" t="n">
+      <c r="I23" t="n">
         <v>14</v>
       </c>
-      <c r="J22" t="n">
+      <c r="J23" t="n">
         <v>7.8</v>
       </c>
-      <c r="L22" t="n">
+      <c r="L23" t="n">
         <v>72.13</v>
       </c>
-      <c r="M22" t="n">
+      <c r="M23" t="n">
         <v>12</v>
       </c>
-      <c r="P22" t="n">
+      <c r="P23" t="n">
         <v>27</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="Q23" t="n">
         <v>-2.1</v>
       </c>
-      <c r="AA22" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="AB22" t="inlineStr">
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
         <is>
           <t>reports/uzbekistan-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-08 17:51
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB23"/>
+  <dimension ref="A1:AB24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1821,6 +1821,69 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Zambia</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Caa2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Concluded 38-month US$1.3bn ECF in Jan-26; negotiating successor program</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="I24" t="n">
+        <v>10.75</v>
+      </c>
+      <c r="J24" t="n">
+        <v>4.65</v>
+      </c>
+      <c r="L24" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="M24" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="P24" t="n">
+        <v>91</v>
+      </c>
+      <c r="S24" t="n">
+        <v>35</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>reports/zambia-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
site build 2026-10-08 18:32
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB24"/>
+  <dimension ref="A1:AB25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1629,61 +1629,50 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>Frozen USD 1.9bn EFF agreed at staff level in Oct-22; no active Executive Board approval</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>29.73</v>
+        <v>5.6</v>
       </c>
       <c r="I21" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="J21" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="K21" t="n">
-        <v>-2.7</v>
-      </c>
-      <c r="L21" t="n">
-        <v>61.56</v>
-      </c>
-      <c r="N21" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="O21" t="n">
-        <v>31.8</v>
+        <v>1.4</v>
+      </c>
+      <c r="M21" t="n">
+        <v>3.1</v>
       </c>
       <c r="P21" t="n">
-        <v>29.5</v>
+        <v>82</v>
       </c>
       <c r="Q21" t="n">
         <v>-5.2</v>
       </c>
+      <c r="X21" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA21" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -1691,14 +1680,14 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/tunisia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1708,41 +1697,50 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>EFF (4-year)</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I22" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J22" t="n">
-        <v>7.9</v>
+        <v>7.27</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-2.7</v>
       </c>
       <c r="L22" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="M22" t="n">
-        <v>5.6</v>
+        <v>61.56</v>
+      </c>
+      <c r="N22" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O22" t="n">
+        <v>31.8</v>
       </c>
       <c r="P22" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>-5.2</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -1751,64 +1749,58 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CIS</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC+</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Ca</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="G23" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year)</t>
+        </is>
       </c>
       <c r="H23" t="n">
-        <v>6.2</v>
+        <v>8.1</v>
       </c>
       <c r="I23" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J23" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="L23" t="n">
-        <v>72.13</v>
+        <v>47.1</v>
       </c>
       <c r="M23" t="n">
-        <v>12</v>
+        <v>5.6</v>
       </c>
       <c r="P23" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q23" t="n">
-        <v>-2.1</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -1817,68 +1809,134 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>reports/uzbekistan-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H24" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I24" t="n">
+        <v>14</v>
+      </c>
+      <c r="J24" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="L24" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="M24" t="n">
+        <v>12</v>
+      </c>
+      <c r="P24" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB24" t="inlineStr">
+        <is>
+          <t>reports/uzbekistan-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Africa</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>CCC+</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Caa2</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Concluded 38-month US$1.3bn ECF in Jan-26; negotiating successor program</t>
         </is>
       </c>
-      <c r="H24" t="n">
+      <c r="H25" t="n">
         <v>6.1</v>
       </c>
-      <c r="I24" t="n">
+      <c r="I25" t="n">
         <v>10.75</v>
       </c>
-      <c r="J24" t="n">
+      <c r="J25" t="n">
         <v>4.65</v>
       </c>
-      <c r="L24" t="n">
+      <c r="L25" t="n">
         <v>5.8</v>
       </c>
-      <c r="M24" t="n">
+      <c r="M25" t="n">
         <v>4.2</v>
       </c>
-      <c r="P24" t="n">
+      <c r="P25" t="n">
         <v>91</v>
       </c>
-      <c r="S24" t="n">
+      <c r="S25" t="n">
         <v>35</v>
       </c>
-      <c r="AA24" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="AB24" t="inlineStr">
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
         <is>
           <t>reports/zambia-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-08 18:53
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB25"/>
+  <dimension ref="A1:AB26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -820,48 +820,60 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Benin</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Post-Financing Assessment (PFA); ECF/EFF/RSF completed Jul-25</t>
-        </is>
+          <t>Blended 42-month EFF/ECF ($638m) and RSF ($200m) completed 25-Feb-26</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>7.5</v>
       </c>
       <c r="H7" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="O7" t="n">
-        <v>30</v>
+        <v>1.25</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-5.5</v>
       </c>
       <c r="P7" t="n">
-        <v>43</v>
+        <v>54</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="R7" t="n">
+        <v>-0.6</v>
       </c>
       <c r="S7" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="T7" t="n">
-        <v>12</v>
+        <v>14.5</v>
+      </c>
+      <c r="X7" t="n">
+        <v>2.85</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
@@ -870,14 +882,14 @@
       </c>
       <c r="AB7" t="inlineStr">
         <is>
-          <t>reports/cameroon-sovereign-credit.md</t>
+          <t>reports/benin-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Cote d'Ivoire</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -887,41 +899,38 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>EFF/ECF ($3.5B) and RSF ($1.3B) completed Jun-26</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>6</v>
+          <t>Post-Financing Assessment (PFA); ECF/EFF/RSF completed Jul-25</t>
+        </is>
       </c>
       <c r="H8" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I8" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" t="n">
-        <v>1.8</v>
+        <v>2.6</v>
+      </c>
+      <c r="O8" t="n">
+        <v>30</v>
       </c>
       <c r="P8" t="n">
-        <v>55.1</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>-3.8</v>
+        <v>43</v>
+      </c>
+      <c r="S8" t="n">
+        <v>20</v>
+      </c>
+      <c r="T8" t="n">
+        <v>12</v>
       </c>
       <c r="AA8" t="inlineStr">
         <is>
@@ -930,61 +939,58 @@
       </c>
       <c r="AB8" t="inlineStr">
         <is>
-          <t>reports/cote-d-ivoire-sovereign-credit.md</t>
+          <t>reports/cameroon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Cote d'Ivoire</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>EFF</t>
-        </is>
+          <t>EFF/ECF ($3.5B) and RSF ($1.3B) completed Jun-26</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>6</v>
       </c>
       <c r="H9" t="n">
-        <v>12.7</v>
+        <v>1.2</v>
       </c>
       <c r="I9" t="n">
-        <v>19</v>
+        <v>3</v>
       </c>
       <c r="J9" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="M9" t="n">
-        <v>7.5</v>
+        <v>1.8</v>
       </c>
       <c r="P9" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="R9" t="n">
-        <v>4</v>
-      </c>
-      <c r="S9" t="n">
-        <v>50</v>
+        <v>55.1</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>-3.8</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
@@ -993,41 +999,61 @@
       </c>
       <c r="AB9" t="inlineStr">
         <is>
-          <t>reports/egypt-sovereign-credit.md</t>
+          <t>reports/cote-d-ivoire-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Gabon</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>CCC-</t>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>B</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>None (technical surveillance only)</t>
-        </is>
+          <t>EFF</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>12.7</v>
+      </c>
+      <c r="I10" t="n">
+        <v>19</v>
+      </c>
+      <c r="J10" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="M10" t="n">
+        <v>7.5</v>
       </c>
       <c r="P10" t="n">
-        <v>70</v>
-      </c>
-      <c r="U10" t="n">
-        <v>17.5</v>
+        <v>79.7</v>
+      </c>
+      <c r="R10" t="n">
+        <v>4</v>
+      </c>
+      <c r="S10" t="n">
+        <v>50</v>
       </c>
       <c r="AA10" t="inlineStr">
         <is>
@@ -1036,14 +1062,14 @@
       </c>
       <c r="AB10" t="inlineStr">
         <is>
-          <t>reports/gabon-sovereign-credit.md</t>
+          <t>reports/egypt-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1053,38 +1079,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>B-</t>
+          <t>CCC-</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="I11" t="n">
-        <v>14</v>
-      </c>
-      <c r="J11" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="L11" t="n">
-        <v>12</v>
-      </c>
-      <c r="M11" t="n">
-        <v>5.2</v>
+          <t>None (technical surveillance only)</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>70</v>
+      </c>
+      <c r="U11" t="n">
+        <v>17.5</v>
       </c>
       <c r="AA11" t="inlineStr">
         <is>
@@ -1093,31 +1105,31 @@
       </c>
       <c r="AB11" t="inlineStr">
         <is>
-          <t>reports/ghana-sovereign-credit.md</t>
+          <t>reports/gabon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
       <c r="E12" t="inlineStr">
         <is>
           <t>Caa1</t>
@@ -1125,20 +1137,23 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>None (Article IV / Post-Financing Assessment)</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
-        <v>-6.8</v>
+          <t>PCI (36-month, non-financing) after ECF $3.0B completed 27-Jul-26</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="I12" t="n">
+        <v>14</v>
+      </c>
+      <c r="J12" t="n">
+        <v>8.800000000000001</v>
       </c>
       <c r="L12" t="n">
-        <v>80.59999999999999</v>
+        <v>12</v>
       </c>
       <c r="M12" t="n">
-        <v>9.6</v>
-      </c>
-      <c r="X12" t="n">
-        <v>0.506</v>
+        <v>5.2</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
@@ -1147,14 +1162,14 @@
       </c>
       <c r="AB12" t="inlineStr">
         <is>
-          <t>reports/iraq-sovereign-credit.md</t>
+          <t>reports/ghana-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -1164,44 +1179,35 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>EFF (4-year) + RSF</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>6</v>
+          <t>None (Article IV / Post-Financing Assessment)</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>-6.8</v>
       </c>
       <c r="L13" t="n">
-        <v>28.5</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M13" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="P13" t="n">
-        <v>83.59999999999999</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="R13" t="n">
-        <v>-2.8</v>
+        <v>9.6</v>
       </c>
       <c r="X13" t="n">
-        <v>3.95</v>
+        <v>0.506</v>
       </c>
       <c r="AA13" t="inlineStr">
         <is>
@@ -1210,61 +1216,61 @@
       </c>
       <c r="AB13" t="inlineStr">
         <is>
-          <t>reports/jordan-sovereign-credit.md</t>
+          <t>reports/iraq-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year) + RSF</t>
+        </is>
       </c>
       <c r="I14" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="J14" t="n">
-        <v>1.95</v>
+        <v>6</v>
       </c>
       <c r="L14" t="n">
-        <v>14.702</v>
+        <v>28.5</v>
+      </c>
+      <c r="M14" t="n">
+        <v>9.199999999999999</v>
       </c>
       <c r="P14" t="n">
-        <v>68.5</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q14" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="S14" t="n">
-        <v>33</v>
+        <v>-5.2</v>
+      </c>
+      <c r="R14" t="n">
+        <v>-2.8</v>
+      </c>
+      <c r="X14" t="n">
+        <v>3.95</v>
       </c>
       <c r="AA14" t="inlineStr">
         <is>
@@ -1273,58 +1279,61 @@
       </c>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>reports/kenya-sovereign-credit.md</t>
+          <t>reports/jordan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Ba1</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>FCL (2-year, precautionary)</t>
-        </is>
+          <t>None (previous EFF/ECF/RSF expired Apr-25; successor under discussion)</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>6.8</v>
       </c>
       <c r="I15" t="n">
-        <v>2.25</v>
+        <v>8.75</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1.95</v>
       </c>
       <c r="L15" t="n">
-        <v>55.65</v>
-      </c>
-      <c r="M15" t="n">
-        <v>5.5</v>
+        <v>14.702</v>
       </c>
       <c r="P15" t="n">
-        <v>66.5</v>
+        <v>68.5</v>
       </c>
       <c r="Q15" t="n">
-        <v>-3</v>
+        <v>-6.4</v>
       </c>
       <c r="S15" t="n">
-        <v>11.5</v>
+        <v>33</v>
       </c>
       <c r="AA15" t="inlineStr">
         <is>
@@ -1333,58 +1342,58 @@
       </c>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>reports/morocco-sovereign-credit.md</t>
+          <t>reports/kenya-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>B3</t>
+          <t>Ba1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>15.39</v>
+          <t>FCL (2-year, precautionary)</t>
+        </is>
       </c>
       <c r="I16" t="n">
-        <v>23</v>
-      </c>
-      <c r="J16" t="n">
-        <v>7.61</v>
+        <v>2.25</v>
       </c>
       <c r="L16" t="n">
-        <v>54.98</v>
+        <v>55.65</v>
+      </c>
+      <c r="M16" t="n">
+        <v>5.5</v>
       </c>
       <c r="P16" t="n">
-        <v>32.3</v>
+        <v>66.5</v>
+      </c>
+      <c r="Q16" t="n">
+        <v>-3</v>
       </c>
       <c r="S16" t="n">
-        <v>55</v>
+        <v>11.5</v>
       </c>
       <c r="AA16" t="inlineStr">
         <is>
@@ -1393,34 +1402,34 @@
       </c>
       <c r="AB16" t="inlineStr">
         <is>
-          <t>reports/nigeria-sovereign-credit.md</t>
+          <t>reports/morocco-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Baa3</t>
+          <t>B3</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1428,20 +1437,23 @@
           <t>None (Article IV)</t>
         </is>
       </c>
-      <c r="G17" t="n">
-        <v>2.1</v>
+      <c r="H17" t="n">
+        <v>15.39</v>
+      </c>
+      <c r="I17" t="n">
+        <v>23</v>
+      </c>
+      <c r="J17" t="n">
+        <v>7.61</v>
       </c>
       <c r="L17" t="n">
-        <v>18.38</v>
-      </c>
-      <c r="M17" t="n">
-        <v>5</v>
+        <v>54.98</v>
       </c>
       <c r="P17" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="Q17" t="n">
-        <v>0.65</v>
+        <v>32.3</v>
+      </c>
+      <c r="S17" t="n">
+        <v>55</v>
       </c>
       <c r="AA17" t="inlineStr">
         <is>
@@ -1450,47 +1462,55 @@
       </c>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>reports/oman-sovereign-credit.md</t>
+          <t>reports/nigeria-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>Baa3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="I18" t="n">
-        <v>3</v>
-      </c>
-      <c r="J18" t="n">
-        <v>1.8</v>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="L18" t="n">
+        <v>18.38</v>
+      </c>
+      <c r="M18" t="n">
+        <v>5</v>
       </c>
       <c r="P18" t="n">
-        <v>132</v>
+        <v>34.7</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0.65</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
@@ -1499,58 +1519,47 @@
       </c>
       <c r="AB18" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/oman-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Europe</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing)</t>
-        </is>
-      </c>
-      <c r="G19" t="n">
-        <v>3.3</v>
+          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
+        </is>
       </c>
       <c r="H19" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I19" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J19" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="K19" t="n">
-        <v>-4.1</v>
+        <v>1.8</v>
       </c>
       <c r="P19" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -1559,29 +1568,29 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -1591,29 +1600,26 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
+          <t>PCI (36-month, non-financing)</t>
+        </is>
+      </c>
+      <c r="G20" t="n">
+        <v>3.3</v>
       </c>
       <c r="H20" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I20" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J20" t="n">
-        <v>2.85</v>
+        <v>3.55</v>
       </c>
       <c r="K20" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="L20" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="M20" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="Q20" t="n">
-        <v>-4.5</v>
+        <v>-4.1</v>
+      </c>
+      <c r="P20" t="n">
+        <v>43.3</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -1622,56 +1628,61 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>BB</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Frozen USD 1.9bn EFF agreed at staff level in Oct-22; no active Executive Board approval</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="I21" t="n">
-        <v>7</v>
+        <v>7.25</v>
       </c>
       <c r="J21" t="n">
-        <v>1.4</v>
+        <v>2.85</v>
+      </c>
+      <c r="K21" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="L21" t="n">
+        <v>63.5</v>
       </c>
       <c r="M21" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P21" t="n">
-        <v>82</v>
+        <v>5.8</v>
       </c>
       <c r="Q21" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="X21" t="n">
-        <v>0.15</v>
+        <v>-4.5</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -1680,68 +1691,57 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>reports/tunisia-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>Frozen USD 1.9bn EFF agreed at staff level in Oct-22; no active Executive Board approval</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>29.73</v>
+        <v>5.6</v>
       </c>
       <c r="I22" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="J22" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="K22" t="n">
-        <v>-2.7</v>
-      </c>
-      <c r="L22" t="n">
-        <v>61.56</v>
-      </c>
-      <c r="N22" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="O22" t="n">
-        <v>31.8</v>
+        <v>1.4</v>
+      </c>
+      <c r="M22" t="n">
+        <v>3.1</v>
       </c>
       <c r="P22" t="n">
-        <v>29.5</v>
+        <v>82</v>
       </c>
       <c r="Q22" t="n">
         <v>-5.2</v>
       </c>
+      <c r="X22" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA22" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -1749,14 +1749,14 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/tunisia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1766,41 +1766,50 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>EFF (4-year)</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I23" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J23" t="n">
-        <v>7.9</v>
+        <v>7.27</v>
+      </c>
+      <c r="K23" t="n">
+        <v>-2.7</v>
       </c>
       <c r="L23" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="M23" t="n">
-        <v>5.6</v>
+        <v>61.56</v>
+      </c>
+      <c r="N23" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O23" t="n">
+        <v>31.8</v>
       </c>
       <c r="P23" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>-5.2</v>
       </c>
       <c r="AA23" t="inlineStr">
         <is>
@@ -1809,64 +1818,58 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CIS</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC+</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Ca</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="G24" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year)</t>
+        </is>
       </c>
       <c r="H24" t="n">
-        <v>6.2</v>
+        <v>8.1</v>
       </c>
       <c r="I24" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J24" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="L24" t="n">
-        <v>72.13</v>
+        <v>47.1</v>
       </c>
       <c r="M24" t="n">
-        <v>12</v>
+        <v>5.6</v>
       </c>
       <c r="P24" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q24" t="n">
-        <v>-2.1</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -1875,68 +1878,134 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>reports/uzbekistan-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H25" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I25" t="n">
+        <v>14</v>
+      </c>
+      <c r="J25" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="L25" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="M25" t="n">
+        <v>12</v>
+      </c>
+      <c r="P25" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB25" t="inlineStr">
+        <is>
+          <t>reports/uzbekistan-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>Africa</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D26" t="inlineStr">
         <is>
           <t>CCC+</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>Caa2</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>Concluded 38-month US$1.3bn ECF in Jan-26; negotiating successor program</t>
         </is>
       </c>
-      <c r="H25" t="n">
+      <c r="H26" t="n">
         <v>6.1</v>
       </c>
-      <c r="I25" t="n">
+      <c r="I26" t="n">
         <v>10.75</v>
       </c>
-      <c r="J25" t="n">
+      <c r="J26" t="n">
         <v>4.65</v>
       </c>
-      <c r="L25" t="n">
+      <c r="L26" t="n">
         <v>5.8</v>
       </c>
-      <c r="M25" t="n">
+      <c r="M26" t="n">
         <v>4.2</v>
       </c>
-      <c r="P25" t="n">
+      <c r="P26" t="n">
         <v>91</v>
       </c>
-      <c r="S25" t="n">
+      <c r="S26" t="n">
         <v>35</v>
       </c>
-      <c r="AA25" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="AB25" t="inlineStr">
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
         <is>
           <t>reports/zambia-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-08 19:10
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB26"/>
+  <dimension ref="A1:AB27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1526,40 +1526,66 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>B+</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>B+</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Caa2</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
-        </is>
+          <t>38-month ECF ($35.7m SDR 26.43m review)</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>7.8</v>
       </c>
       <c r="H19" t="n">
-        <v>1.2</v>
+        <v>15.7</v>
       </c>
       <c r="I19" t="n">
-        <v>3</v>
+        <v>8.75</v>
       </c>
       <c r="J19" t="n">
-        <v>1.8</v>
+        <v>-6.95</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-15</v>
+      </c>
+      <c r="L19" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="M19" t="n">
+        <v>4</v>
+      </c>
+      <c r="O19" t="n">
+        <v>63</v>
       </c>
       <c r="P19" t="n">
-        <v>132</v>
+        <v>77.5</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>-4.8</v>
+      </c>
+      <c r="X19" t="n">
+        <v>0.62</v>
       </c>
       <c r="AA19" t="inlineStr">
         <is>
@@ -1568,58 +1594,47 @@
       </c>
       <c r="AB19" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/rwanda-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Europe</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>PCI (36-month, non-financing)</t>
-        </is>
-      </c>
-      <c r="G20" t="n">
-        <v>3.3</v>
+          <t>Staff-level agreement on successor arrangement (replaces suspended $1.8B facility)</t>
+        </is>
       </c>
       <c r="H20" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I20" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J20" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="K20" t="n">
-        <v>-4.1</v>
+        <v>1.8</v>
       </c>
       <c r="P20" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="AA20" t="inlineStr">
         <is>
@@ -1628,29 +1643,29 @@
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1660,29 +1675,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
+          <t>PCI (36-month, non-financing)</t>
+        </is>
+      </c>
+      <c r="G21" t="n">
+        <v>3.3</v>
       </c>
       <c r="H21" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I21" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J21" t="n">
-        <v>2.85</v>
+        <v>3.55</v>
       </c>
       <c r="K21" t="n">
-        <v>-1.6</v>
-      </c>
-      <c r="L21" t="n">
-        <v>63.5</v>
-      </c>
-      <c r="M21" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>-4.5</v>
+        <v>-4.1</v>
+      </c>
+      <c r="P21" t="n">
+        <v>43.3</v>
       </c>
       <c r="AA21" t="inlineStr">
         <is>
@@ -1691,56 +1703,61 @@
       </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Middle East</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>BB</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Caa1</t>
+          <t>Ba2</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Frozen USD 1.9bn EFF agreed at staff level in Oct-22; no active Executive Board approval</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>5.6</v>
+        <v>4.4</v>
       </c>
       <c r="I22" t="n">
-        <v>7</v>
+        <v>7.25</v>
       </c>
       <c r="J22" t="n">
-        <v>1.4</v>
+        <v>2.85</v>
+      </c>
+      <c r="K22" t="n">
+        <v>-1.6</v>
+      </c>
+      <c r="L22" t="n">
+        <v>63.5</v>
       </c>
       <c r="M22" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="P22" t="n">
-        <v>82</v>
+        <v>5.8</v>
       </c>
       <c r="Q22" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="X22" t="n">
-        <v>0.15</v>
+        <v>-4.5</v>
       </c>
       <c r="AA22" t="inlineStr">
         <is>
@@ -1749,68 +1766,57 @@
       </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>reports/tunisia-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Middle East</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Ba3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>Frozen USD 1.9bn EFF agreed at staff level in Oct-22; no active Executive Board approval</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>29.73</v>
+        <v>5.6</v>
       </c>
       <c r="I23" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="J23" t="n">
-        <v>7.27</v>
-      </c>
-      <c r="K23" t="n">
-        <v>-2.7</v>
-      </c>
-      <c r="L23" t="n">
-        <v>61.56</v>
-      </c>
-      <c r="N23" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="O23" t="n">
-        <v>31.8</v>
+        <v>1.4</v>
+      </c>
+      <c r="M23" t="n">
+        <v>3.1</v>
       </c>
       <c r="P23" t="n">
-        <v>29.5</v>
+        <v>82</v>
       </c>
       <c r="Q23" t="n">
         <v>-5.2</v>
       </c>
+      <c r="X23" t="n">
+        <v>0.15</v>
+      </c>
       <c r="AA23" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -1818,14 +1824,14 @@
       </c>
       <c r="AB23" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/tunisia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1835,41 +1841,50 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Ca</t>
+          <t>Ba3</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>EFF (4-year)</t>
+          <t>None (Article IV)</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I24" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J24" t="n">
-        <v>7.9</v>
+        <v>7.27</v>
+      </c>
+      <c r="K24" t="n">
+        <v>-2.7</v>
       </c>
       <c r="L24" t="n">
-        <v>47.1</v>
-      </c>
-      <c r="M24" t="n">
-        <v>5.6</v>
+        <v>61.56</v>
+      </c>
+      <c r="N24" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="O24" t="n">
+        <v>31.8</v>
       </c>
       <c r="P24" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>-5.2</v>
       </c>
       <c r="AA24" t="inlineStr">
         <is>
@@ -1878,64 +1893,58 @@
       </c>
       <c r="AB24" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CIS</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>CCC+</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Ca</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
-        </is>
-      </c>
-      <c r="G25" t="n">
-        <v>6.8</v>
+          <t>EFF (4-year)</t>
+        </is>
       </c>
       <c r="H25" t="n">
-        <v>6.2</v>
+        <v>8.1</v>
       </c>
       <c r="I25" t="n">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="J25" t="n">
-        <v>7.8</v>
+        <v>7.9</v>
       </c>
       <c r="L25" t="n">
-        <v>72.13</v>
+        <v>47.1</v>
       </c>
       <c r="M25" t="n">
-        <v>12</v>
+        <v>5.6</v>
       </c>
       <c r="P25" t="n">
-        <v>27</v>
-      </c>
-      <c r="Q25" t="n">
-        <v>-2.1</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="AA25" t="inlineStr">
         <is>
@@ -1944,68 +1953,134 @@
       </c>
       <c r="AB25" t="inlineStr">
         <is>
-          <t>reports/uzbekistan-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CIS</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H26" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I26" t="n">
+        <v>14</v>
+      </c>
+      <c r="J26" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="L26" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="M26" t="n">
+        <v>12</v>
+      </c>
+      <c r="P26" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>reports/uzbekistan-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Africa</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr">
+      <c r="D27" t="inlineStr">
         <is>
           <t>CCC+</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Caa2</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>Concluded 38-month US$1.3bn ECF in Jan-26; negotiating successor program</t>
         </is>
       </c>
-      <c r="H26" t="n">
+      <c r="H27" t="n">
         <v>6.1</v>
       </c>
-      <c r="I26" t="n">
+      <c r="I27" t="n">
         <v>10.75</v>
       </c>
-      <c r="J26" t="n">
+      <c r="J27" t="n">
         <v>4.65</v>
       </c>
-      <c r="L26" t="n">
+      <c r="L27" t="n">
         <v>5.8</v>
       </c>
-      <c r="M26" t="n">
+      <c r="M27" t="n">
         <v>4.2</v>
       </c>
-      <c r="P26" t="n">
+      <c r="P27" t="n">
         <v>91</v>
       </c>
-      <c r="S26" t="n">
+      <c r="S27" t="n">
         <v>35</v>
       </c>
-      <c r="AA26" t="inlineStr">
-        <is>
-          <t>08-Oct-26</t>
-        </is>
-      </c>
-      <c r="AB26" t="inlineStr">
+      <c r="AA27" t="inlineStr">
+        <is>
+          <t>08-Oct-26</t>
+        </is>
+      </c>
+      <c r="AB27" t="inlineStr">
         <is>
           <t>reports/zambia-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-08 21:06
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -3528,13 +3528,13 @@
         <v>-2.7</v>
       </c>
       <c r="L47" t="n">
-        <v>61.56</v>
+        <v>174.4</v>
       </c>
       <c r="M47" t="n">
         <v>5.128</v>
       </c>
       <c r="N47" t="n">
-        <v>0.36</v>
+        <v>1.02</v>
       </c>
       <c r="O47" t="n">
         <v>31.8</v>

</xml_diff>

<commit_message>
site build 2026-10-08 21:16
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -2623,6 +2623,12 @@
       <c r="Y31" t="n">
         <v>-6.3</v>
       </c>
+      <c r="Z31" t="n">
+        <v>2.151</v>
+      </c>
+      <c r="AA31" t="n">
+        <v>-1.86</v>
+      </c>
       <c r="AB31" t="n">
         <v>0.8</v>
       </c>
@@ -2700,6 +2706,9 @@
       <c r="Y32" t="n">
         <v>30.8</v>
       </c>
+      <c r="AA32" t="n">
+        <v>15.61</v>
+      </c>
       <c r="AB32" t="n">
         <v>4.6</v>
       </c>
@@ -2775,6 +2784,12 @@
       </c>
       <c r="Y33" t="n">
         <v>7.2</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>4.474</v>
+      </c>
+      <c r="AA33" t="n">
+        <v>-0.99</v>
       </c>
       <c r="AB33" t="n">
         <v>-2.6</v>
@@ -2901,6 +2916,9 @@
       <c r="Y35" t="n">
         <v>22.8</v>
       </c>
+      <c r="AA35" t="n">
+        <v>-0.14</v>
+      </c>
       <c r="AB35" t="n">
         <v>-2.3</v>
       </c>
@@ -2955,6 +2973,12 @@
       <c r="Y36" t="n">
         <v>16.3</v>
       </c>
+      <c r="Z36" t="n">
+        <v>87.288</v>
+      </c>
+      <c r="AA36" t="n">
+        <v>12.01</v>
+      </c>
       <c r="AB36" t="n">
         <v>2.5</v>
       </c>
@@ -3009,6 +3033,12 @@
       <c r="Y37" t="n">
         <v>-2</v>
       </c>
+      <c r="Z37" t="n">
+        <v>93.018</v>
+      </c>
+      <c r="AA37" t="n">
+        <v>-22.11</v>
+      </c>
       <c r="AB37" t="n">
         <v>-1.4</v>
       </c>
@@ -3063,6 +3093,12 @@
       <c r="Y38" t="n">
         <v>16.9</v>
       </c>
+      <c r="Z38" t="n">
+        <v>277.21</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>-13.87</v>
+      </c>
       <c r="AB38" t="n">
         <v>-1.1</v>
       </c>
@@ -3117,6 +3153,12 @@
       <c r="Y39" t="n">
         <v>2.9</v>
       </c>
+      <c r="Z39" t="n">
+        <v>72.172</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>-32.2</v>
+      </c>
       <c r="AB39" t="n">
         <v>-0.5</v>
       </c>
@@ -3195,6 +3237,12 @@
       <c r="Y40" t="n">
         <v>-16.4</v>
       </c>
+      <c r="Z40" t="n">
+        <v>1.795</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>-1.98</v>
+      </c>
       <c r="AB40" t="n">
         <v>-0</v>
       </c>
@@ -3340,6 +3388,12 @@
       <c r="Y42" t="n">
         <v>7</v>
       </c>
+      <c r="Z42" t="n">
+        <v>30.033</v>
+      </c>
+      <c r="AA42" t="n">
+        <v>-4.36</v>
+      </c>
       <c r="AB42" t="n">
         <v>-1.4</v>
       </c>
@@ -3420,6 +3474,12 @@
       </c>
       <c r="Y43" t="n">
         <v>7.8</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>74.307</v>
+      </c>
+      <c r="AA43" t="n">
+        <v>-1.32</v>
       </c>
       <c r="AB43" t="n">
         <v>-0.9</v>
@@ -3471,6 +3531,9 @@
       <c r="Y44" t="n">
         <v>45.9</v>
       </c>
+      <c r="AA44" t="n">
+        <v>3.48</v>
+      </c>
       <c r="AB44" t="n">
         <v>-0.8</v>
       </c>
@@ -3525,6 +3588,12 @@
       <c r="Y45" t="n">
         <v>5.9</v>
       </c>
+      <c r="Z45" t="n">
+        <v>302.852</v>
+      </c>
+      <c r="AA45" t="n">
+        <v>8.08</v>
+      </c>
       <c r="AB45" t="n">
         <v>-3.9</v>
       </c>
@@ -3597,6 +3666,9 @@
       </c>
       <c r="Y46" t="n">
         <v>6.8</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>-1.33</v>
       </c>
       <c r="AB46" t="n">
         <v>-1.2</v>
@@ -3765,6 +3837,12 @@
       <c r="Y48" t="n">
         <v>5.7</v>
       </c>
+      <c r="Z48" t="n">
+        <v>38.646</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>-24.81</v>
+      </c>
       <c r="AB48" t="n">
         <v>-2.3</v>
       </c>
@@ -3840,6 +3918,9 @@
       <c r="Y49" t="n">
         <v>32</v>
       </c>
+      <c r="AA49" t="n">
+        <v>-11.23</v>
+      </c>
       <c r="AF49" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -3917,6 +3998,9 @@
       </c>
       <c r="Y50" t="n">
         <v>25.6</v>
+      </c>
+      <c r="AA50" t="n">
+        <v>-0.9</v>
       </c>
       <c r="AB50" t="n">
         <v>5.1</v>

</xml_diff>

<commit_message>
site build 2026-10-08 21:26
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -1062,6 +1062,11 @@
           <t>Brazil</t>
         </is>
       </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="n">
         <v>1.9</v>
@@ -1206,6 +1211,11 @@
           <t>Chile</t>
         </is>
       </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="n">
         <v>2.4</v>
@@ -1266,6 +1276,11 @@
           <t>Colombia</t>
         </is>
       </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="n">
         <v>2.3</v>
@@ -1395,6 +1410,11 @@
           <t>Czech Republic</t>
         </is>
       </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Central Europe</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="n">
         <v>2.2</v>
@@ -1836,6 +1856,11 @@
           <t>Hungary</t>
         </is>
       </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Central Europe</t>
+        </is>
+      </c>
       <c r="F20" t="inlineStr"/>
       <c r="G20" t="n">
         <v>1.7</v>
@@ -1896,6 +1921,11 @@
           <t>India</t>
         </is>
       </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
         <v>6.5</v>
@@ -1956,6 +1986,11 @@
           <t>Indonesia</t>
         </is>
       </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
         <v>5</v>
@@ -2256,6 +2291,11 @@
           <t>Malaysia</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
         <v>4.7</v>
@@ -2316,6 +2356,11 @@
           <t>Mexico</t>
         </is>
       </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
       <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
         <v>1.6</v>
@@ -2946,6 +2991,11 @@
           <t>Peru</t>
         </is>
       </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Latin America</t>
+        </is>
+      </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
         <v>2.8</v>
@@ -3006,6 +3056,11 @@
           <t>Philippines</t>
         </is>
       </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Asia</t>
+        </is>
+      </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
         <v>4.1</v>
@@ -3066,6 +3121,11 @@
           <t>Poland</t>
         </is>
       </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Central Europe</t>
+        </is>
+      </c>
       <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
         <v>3.3</v>
@@ -3126,6 +3186,11 @@
           <t>Romania</t>
         </is>
       </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Central Europe</t>
+        </is>
+      </c>
       <c r="F39" t="inlineStr"/>
       <c r="G39" t="n">
         <v>0.7</v>
@@ -3559,6 +3624,11 @@
       <c r="A45" t="inlineStr">
         <is>
           <t>Thailand</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Asia</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>

</xml_diff>

<commit_message>
site build 2026-10-09 07:00
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -2160,6 +2160,12 @@
       <c r="Y24" t="n">
         <v>4.9</v>
       </c>
+      <c r="Z24" t="n">
+        <v>232.204</v>
+      </c>
+      <c r="AA24" t="n">
+        <v>4.53</v>
+      </c>
       <c r="AB24" t="n">
         <v>-1.6</v>
       </c>
@@ -2292,6 +2298,12 @@
       <c r="Y26" t="n">
         <v>29.9</v>
       </c>
+      <c r="Z26" t="n">
+        <v>59.792</v>
+      </c>
+      <c r="AA26" t="n">
+        <v>-13.41</v>
+      </c>
       <c r="AB26" t="n">
         <v>11.5</v>
       </c>
@@ -2417,6 +2429,9 @@
       <c r="Y28" t="n">
         <v>-23.4</v>
       </c>
+      <c r="AA28" t="n">
+        <v>32.54</v>
+      </c>
       <c r="AB28" t="n">
         <v>28.1</v>
       </c>
@@ -2462,6 +2477,9 @@
       <c r="Y29" t="n">
         <v>31.2</v>
       </c>
+      <c r="AA29" t="n">
+        <v>-9.16</v>
+      </c>
       <c r="AB29" t="n">
         <v>-4.6</v>
       </c>
@@ -3408,6 +3426,9 @@
       <c r="Y43" t="n">
         <v>10.4</v>
       </c>
+      <c r="AA43" t="n">
+        <v>28.52</v>
+      </c>
       <c r="AB43" t="n">
         <v>14.7</v>
       </c>
@@ -3613,6 +3634,12 @@
       </c>
       <c r="Y46" t="n">
         <v>10</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>482.147</v>
+      </c>
+      <c r="AA46" t="n">
+        <v>-25.78</v>
       </c>
       <c r="AB46" t="n">
         <v>15.9</v>

</xml_diff>

<commit_message>
site build 2026-10-09 07:02
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -2126,6 +2126,11 @@
           <t>Israel</t>
         </is>
       </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Middle East (EMBI IG)</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
         <v>3.5</v>
@@ -2273,6 +2278,11 @@
           <t>Kazakhstan</t>
         </is>
       </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>CIS / Central Asia (EMBI IG)</t>
+        </is>
+      </c>
       <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
         <v>4.6</v>
@@ -2398,6 +2408,11 @@
           <t>Kuwait</t>
         </is>
       </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>MENA / GCC (EMBI IG)</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
         <v>-0.6</v>
@@ -2452,6 +2467,11 @@
           <t>Lebanon</t>
         </is>
       </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Middle East (EMBI, in default since 2020)</t>
+        </is>
+      </c>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
         <v>4</v>
@@ -3395,6 +3415,11 @@
           <t>Qatar</t>
         </is>
       </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>MENA / GCC (EMBI IG)</t>
+        </is>
+      </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
         <v>-8.6</v>
@@ -3601,6 +3626,11 @@
           <t>Saudi Arabia</t>
         </is>
       </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MENA / GCC (EMBI IG)</t>
+        </is>
+      </c>
       <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
         <v>3.1</v>
@@ -4177,6 +4207,11 @@
       <c r="A54" t="inlineStr">
         <is>
           <t>Uae</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>MENA / GCC (EMBI IG)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>

</xml_diff>

<commit_message>
site build 2026-10-09 07:28
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -4210,44 +4210,75 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Uae</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MENA / GCC (EMBI IG)</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
+          <t>CEEMEA</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>CCC</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>4-year EFF</t>
+        </is>
+      </c>
       <c r="G54" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="H54" t="n">
-        <v>2.0488</v>
+        <v>8.1</v>
+      </c>
+      <c r="I54" t="n">
+        <v>16</v>
+      </c>
+      <c r="J54" t="n">
+        <v>7.9</v>
       </c>
       <c r="K54" t="n">
-        <v>11.4</v>
+        <v>-18.9</v>
       </c>
       <c r="L54" t="n">
-        <v>259.72</v>
+        <v>47.1</v>
       </c>
       <c r="M54" t="n">
-        <v>5.234</v>
+        <v>5.6</v>
       </c>
       <c r="P54" t="n">
-        <v>31.4</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="Q54" t="n">
-        <v>4.9</v>
+        <v>-18.4</v>
       </c>
       <c r="X54" t="n">
-        <v>-1.12</v>
+        <v>-0.5</v>
       </c>
       <c r="Y54" t="n">
-        <v>-3.1</v>
+        <v>5.7</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>38.646</v>
+      </c>
+      <c r="AA54" t="n">
+        <v>-24.81</v>
       </c>
       <c r="AB54" t="n">
-        <v>13.2</v>
+        <v>-2.3</v>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
@@ -4256,82 +4287,61 @@
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>reports/uae-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CEEMEA</t>
+          <t>GCC / Middle East</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>AA-</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CCC+</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>4-year EFF</t>
-        </is>
-      </c>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>2</v>
+        <v>3.1</v>
       </c>
       <c r="H55" t="n">
-        <v>8.1</v>
-      </c>
-      <c r="I55" t="n">
-        <v>16</v>
-      </c>
-      <c r="J55" t="n">
-        <v>7.9</v>
+        <v>2.05</v>
       </c>
       <c r="K55" t="n">
-        <v>-18.9</v>
+        <v>11.4</v>
       </c>
       <c r="L55" t="n">
-        <v>47.1</v>
+        <v>259.7</v>
       </c>
       <c r="M55" t="n">
-        <v>5.6</v>
+        <v>5.2</v>
       </c>
       <c r="P55" t="n">
-        <v>98.40000000000001</v>
+        <v>31.4</v>
       </c>
       <c r="Q55" t="n">
-        <v>-18.4</v>
+        <v>4.9</v>
       </c>
       <c r="X55" t="n">
-        <v>-0.5</v>
+        <v>-1.12</v>
       </c>
       <c r="Y55" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="Z55" t="n">
-        <v>38.646</v>
-      </c>
-      <c r="AA55" t="n">
-        <v>-24.81</v>
+        <v>-3.1</v>
       </c>
       <c r="AB55" t="n">
-        <v>-2.3</v>
+        <v>13.2</v>
       </c>
       <c r="AF55" t="inlineStr">
         <is>
@@ -4340,7 +4350,7 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/uae-sovereign-credit.md</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
site build 2026-10-09 08:33
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG57"/>
+  <dimension ref="A1:AG58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -605,7 +605,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CEEMEA (Balkans)</t>
+          <t>CEEMEA - Southeast Europe (Western Balkans)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -753,7 +753,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Caucasus</t>
+          <t>CEEMEA - South Caucasus</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -773,7 +773,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>3-year precautionary Stand-By Arrangement</t>
+          <t>3-year Stand-By Arrangement (precautionary)</t>
         </is>
       </c>
       <c r="G5" t="n">
@@ -1475,79 +1475,15 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>EM sovereign issuance, index flows and positioning</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MENA</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>EFF (with RSF)</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="H15" t="n">
-        <v>12.7</v>
-      </c>
-      <c r="I15" t="n">
-        <v>19</v>
-      </c>
-      <c r="J15" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="K15" t="n">
-        <v>-4.2</v>
-      </c>
-      <c r="L15" t="n">
-        <v>53.559</v>
-      </c>
-      <c r="M15" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="P15" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="Q15" t="n">
-        <v>-12.1</v>
-      </c>
-      <c r="R15" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="S15" t="n">
-        <v>50</v>
-      </c>
-      <c r="Y15" t="n">
-        <v>14.7</v>
-      </c>
-      <c r="Z15" t="n">
-        <v>17.224</v>
-      </c>
-      <c r="AA15" t="n">
-        <v>-16.76</v>
-      </c>
-      <c r="AB15" t="n">
-        <v>-0.7</v>
-      </c>
+          <t>EM cross-region (thematic, no single country)</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="AF15" t="inlineStr">
         <is>
           <t>09-Oct-26</t>
@@ -1555,76 +1491,85 @@
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>reports/egypt-sovereign-credit.md</t>
+          <t>reports/em-issuance-index-flows-and-positioning-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>MENA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>RD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>SD</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Caa3</t>
+          <t>Caa1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>48-month Extended Credit Facility (ECF)</t>
+          <t>EFF (with RSF)</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>9.199999999999999</v>
+        <v>4.2</v>
       </c>
       <c r="H16" t="n">
-        <v>13.4</v>
+        <v>12.7</v>
+      </c>
+      <c r="I16" t="n">
+        <v>19</v>
+      </c>
+      <c r="J16" t="n">
+        <v>6.3</v>
       </c>
       <c r="K16" t="n">
-        <v>-2.4</v>
+        <v>-4.2</v>
       </c>
       <c r="L16" t="n">
-        <v>3.784</v>
+        <v>53.559</v>
       </c>
       <c r="M16" t="n">
-        <v>1.781</v>
+        <v>7.5</v>
       </c>
       <c r="P16" t="n">
-        <v>40.4</v>
+        <v>79.7</v>
       </c>
       <c r="Q16" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="T16" t="n">
-        <v>7</v>
+        <v>-12.1</v>
+      </c>
+      <c r="R16" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="S16" t="n">
+        <v>50</v>
       </c>
       <c r="Y16" t="n">
-        <v>86.59999999999999</v>
+        <v>14.7</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>17.224</v>
       </c>
       <c r="AA16" t="n">
-        <v>-3.79</v>
+        <v>-16.76</v>
       </c>
       <c r="AB16" t="n">
-        <v>-2.8</v>
-      </c>
-      <c r="AC16" t="n">
-        <v>1</v>
+        <v>-0.7</v>
       </c>
       <c r="AF16" t="inlineStr">
         <is>
@@ -1633,64 +1578,76 @@
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>reports/ethiopia-sovereign-credit.md</t>
+          <t>reports/egypt-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Gabon</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa (CEMAC)</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>CCC-</t>
+          <t>RD</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SD</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Caa2</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr"/>
+          <t>Caa3</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>48-month Extended Credit Facility (ECF)</t>
+        </is>
+      </c>
       <c r="G17" t="n">
-        <v>2.7</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="H17" t="n">
-        <v>1.597</v>
+        <v>13.4</v>
       </c>
       <c r="K17" t="n">
-        <v>-4.3</v>
+        <v>-2.4</v>
       </c>
       <c r="L17" t="n">
-        <v>0.673</v>
+        <v>3.784</v>
       </c>
       <c r="M17" t="n">
-        <v>4.247</v>
+        <v>1.781</v>
       </c>
       <c r="P17" t="n">
-        <v>70</v>
+        <v>40.4</v>
       </c>
       <c r="Q17" t="n">
-        <v>-10</v>
-      </c>
-      <c r="U17" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="X17" t="n">
-        <v>0.6899999999999999</v>
+        <v>-1.8</v>
+      </c>
+      <c r="T17" t="n">
+        <v>7</v>
       </c>
       <c r="Y17" t="n">
-        <v>-51.4</v>
+        <v>86.59999999999999</v>
+      </c>
+      <c r="AA17" t="n">
+        <v>-3.79</v>
       </c>
       <c r="AB17" t="n">
-        <v>22.6</v>
+        <v>-2.8</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>1</v>
       </c>
       <c r="AF17" t="inlineStr">
         <is>
@@ -1699,63 +1656,64 @@
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>reports/gabon-sovereign-credit.md</t>
+          <t>reports/ethiopia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Caucasus</t>
+          <t>Sub-Saharan Africa (CEMAC)</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>CCC-</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="n">
-        <v>5.3</v>
+        <v>2.7</v>
       </c>
       <c r="H18" t="n">
-        <v>5.6478</v>
-      </c>
-      <c r="I18" t="n">
-        <v>8.25</v>
-      </c>
-      <c r="J18" t="n">
-        <v>2.6</v>
+        <v>1.597</v>
       </c>
       <c r="K18" t="n">
-        <v>-5</v>
+        <v>-4.3</v>
       </c>
       <c r="L18" t="n">
-        <v>8.138999999999999</v>
+        <v>0.673</v>
       </c>
       <c r="M18" t="n">
-        <v>3.017</v>
+        <v>4.247</v>
       </c>
       <c r="P18" t="n">
-        <v>35.1</v>
+        <v>70</v>
       </c>
       <c r="Q18" t="n">
-        <v>-2.3</v>
+        <v>-10</v>
+      </c>
+      <c r="U18" t="n">
+        <v>17.5</v>
       </c>
       <c r="X18" t="n">
-        <v>1.22</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="Y18" t="n">
-        <v>56.4</v>
-      </c>
-      <c r="Z18" t="n">
-        <v>7.255</v>
-      </c>
-      <c r="AA18" t="n">
-        <v>-0.72</v>
+        <v>-51.4</v>
       </c>
       <c r="AB18" t="n">
-        <v>-2.5</v>
+        <v>22.6</v>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
@@ -1764,79 +1722,63 @@
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>reports/georgia-sovereign-credit.md</t>
+          <t>reports/gabon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Georgia</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>36-month non-financing Policy Coordination Instrument (PCI), following completion of the US$3.0B ECF</t>
-        </is>
-      </c>
+          <t>Caucasus</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
       <c r="G19" t="n">
-        <v>4.8</v>
+        <v>5.3</v>
       </c>
       <c r="H19" t="n">
-        <v>5.2</v>
+        <v>5.6478</v>
       </c>
       <c r="I19" t="n">
-        <v>14</v>
+        <v>8.25</v>
       </c>
       <c r="J19" t="n">
-        <v>8.800000000000001</v>
+        <v>2.6</v>
       </c>
       <c r="K19" t="n">
-        <v>10.1</v>
+        <v>-5</v>
       </c>
       <c r="L19" t="n">
-        <v>12</v>
+        <v>8.138999999999999</v>
       </c>
       <c r="M19" t="n">
-        <v>5.2</v>
+        <v>3.017</v>
       </c>
       <c r="P19" t="n">
-        <v>53</v>
+        <v>35.1</v>
       </c>
       <c r="Q19" t="n">
         <v>-2.3</v>
       </c>
       <c r="X19" t="n">
-        <v>1.86</v>
+        <v>1.22</v>
       </c>
       <c r="Y19" t="n">
-        <v>11.9</v>
+        <v>56.4</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>7.255</v>
       </c>
       <c r="AA19" t="n">
-        <v>10.06</v>
+        <v>-0.72</v>
       </c>
       <c r="AB19" t="n">
-        <v>3.3</v>
+        <v>-2.5</v>
       </c>
       <c r="AF19" t="inlineStr">
         <is>
@@ -1845,128 +1787,144 @@
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>reports/ghana-sovereign-credit.md</t>
+          <t>reports/georgia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Central Europe</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Caa1</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>36-month non-financing Policy Coordination Instrument (PCI), following completion of the US$3.0B ECF</t>
+        </is>
+      </c>
       <c r="G20" t="n">
-        <v>1.7</v>
+        <v>4.8</v>
       </c>
       <c r="H20" t="n">
-        <v>1.2826</v>
+        <v>5.2</v>
       </c>
       <c r="I20" t="n">
-        <v>5.5</v>
+        <v>14</v>
       </c>
       <c r="J20" t="n">
-        <v>4.22</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K20" t="n">
-        <v>-0.4</v>
+        <v>10.1</v>
       </c>
       <c r="L20" t="n">
-        <v>73.621</v>
+        <v>12</v>
       </c>
       <c r="M20" t="n">
-        <v>3.495</v>
+        <v>5.2</v>
       </c>
       <c r="P20" t="n">
-        <v>77.90000000000001</v>
+        <v>53</v>
       </c>
       <c r="Q20" t="n">
-        <v>-5.5</v>
+        <v>-2.3</v>
       </c>
       <c r="X20" t="n">
-        <v>2.27</v>
+        <v>1.86</v>
       </c>
       <c r="Y20" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="Z20" t="n">
-        <v>66.95</v>
+        <v>11.9</v>
       </c>
       <c r="AA20" t="n">
-        <v>2.37</v>
+        <v>10.06</v>
       </c>
       <c r="AB20" t="n">
-        <v>-1.1</v>
+        <v>3.3</v>
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>reports/hungary-sovereign-credit.md</t>
+          <t>reports/ghana-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Central Europe</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="n">
-        <v>6.5</v>
+        <v>1.7</v>
       </c>
       <c r="H21" t="n">
-        <v>4.4412</v>
+        <v>1.2826</v>
       </c>
       <c r="I21" t="n">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
       <c r="J21" t="n">
-        <v>0.8100000000000001</v>
+        <v>4.22</v>
       </c>
       <c r="K21" t="n">
-        <v>-2</v>
+        <v>-0.4</v>
       </c>
       <c r="L21" t="n">
-        <v>751.764</v>
+        <v>73.621</v>
       </c>
       <c r="M21" t="n">
-        <v>7.851</v>
+        <v>3.495</v>
       </c>
       <c r="P21" t="n">
-        <v>83.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="Q21" t="n">
-        <v>-7.4</v>
+        <v>-5.5</v>
       </c>
       <c r="X21" t="n">
-        <v>-2.75</v>
+        <v>2.27</v>
       </c>
       <c r="Y21" t="n">
-        <v>8.1</v>
+        <v>30.3</v>
       </c>
       <c r="Z21" t="n">
-        <v>715.745</v>
+        <v>66.95</v>
       </c>
       <c r="AA21" t="n">
-        <v>-28.25</v>
+        <v>2.37</v>
       </c>
       <c r="AB21" t="n">
-        <v>-2.8</v>
+        <v>-1.1</v>
       </c>
       <c r="AF21" t="inlineStr">
         <is>
@@ -1975,14 +1933,14 @@
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>reports/india-sovereign-credit.md</t>
+          <t>reports/hungary-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1992,47 +1950,47 @@
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="H22" t="n">
-        <v>2.8821</v>
+        <v>4.4412</v>
       </c>
       <c r="I22" t="n">
-        <v>5.75</v>
+        <v>5.25</v>
       </c>
       <c r="J22" t="n">
-        <v>2.87</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K22" t="n">
-        <v>-1.1</v>
+        <v>-2</v>
       </c>
       <c r="L22" t="n">
-        <v>146.492</v>
+        <v>751.764</v>
       </c>
       <c r="M22" t="n">
-        <v>5.514</v>
+        <v>7.851</v>
       </c>
       <c r="P22" t="n">
-        <v>41.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="Q22" t="n">
-        <v>-2.9</v>
+        <v>-7.4</v>
       </c>
       <c r="X22" t="n">
-        <v>-3.03</v>
+        <v>-2.75</v>
       </c>
       <c r="Y22" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>715.745</v>
+      </c>
+      <c r="AA22" t="n">
+        <v>-28.25</v>
+      </c>
+      <c r="AB22" t="n">
         <v>-2.8</v>
       </c>
-      <c r="Z22" t="n">
-        <v>75.541</v>
-      </c>
-      <c r="AA22" t="n">
-        <v>-14.36</v>
-      </c>
-      <c r="AB22" t="n">
-        <v>0.4</v>
-      </c>
       <c r="AF22" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -2040,138 +1998,138 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>reports/indonesia-sovereign-credit.md</t>
+          <t>reports/india-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>MENA</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>None active (Article IV surveillance and Post-Financing Assessment; last SBA expired 2018)</t>
-        </is>
-      </c>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
-        <v>-6.8</v>
+        <v>5</v>
       </c>
       <c r="H23" t="n">
-        <v>3.0928</v>
+        <v>2.8821</v>
+      </c>
+      <c r="I23" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="J23" t="n">
+        <v>2.87</v>
       </c>
       <c r="K23" t="n">
-        <v>-5.3</v>
+        <v>-1.1</v>
       </c>
       <c r="L23" t="n">
-        <v>80.59999999999999</v>
+        <v>146.492</v>
       </c>
       <c r="M23" t="n">
-        <v>9.6</v>
+        <v>5.514</v>
       </c>
       <c r="P23" t="n">
-        <v>57</v>
+        <v>41.5</v>
       </c>
       <c r="Q23" t="n">
-        <v>-4.2</v>
+        <v>-2.9</v>
+      </c>
+      <c r="X23" t="n">
+        <v>-3.03</v>
       </c>
       <c r="Y23" t="n">
-        <v>-10.9</v>
+        <v>-2.8</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>75.541</v>
       </c>
       <c r="AA23" t="n">
-        <v>4.92</v>
+        <v>-14.36</v>
       </c>
       <c r="AB23" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="AC23" t="n">
-        <v>0.50625</v>
+        <v>0.4</v>
       </c>
       <c r="AF23" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>reports/iraq-sovereign-credit.md</t>
+          <t>reports/indonesia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Middle East</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Caa1</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>None active (Article IV surveillance and Post-Financing Assessment; last SBA expired 2018)</t>
+        </is>
+      </c>
       <c r="G24" t="n">
-        <v>3.5</v>
+        <v>-6.8</v>
       </c>
       <c r="H24" t="n">
-        <v>1.54</v>
-      </c>
-      <c r="I24" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="J24" t="n">
-        <v>1.71</v>
+        <v>3.0928</v>
       </c>
       <c r="K24" t="n">
-        <v>1.9</v>
+        <v>-5.3</v>
       </c>
       <c r="L24" t="n">
-        <v>241.63</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M24" t="n">
-        <v>14.36</v>
+        <v>9.6</v>
       </c>
       <c r="P24" t="n">
-        <v>69.8</v>
+        <v>57</v>
       </c>
       <c r="Q24" t="n">
-        <v>-5.9</v>
-      </c>
-      <c r="X24" t="n">
-        <v>2.67</v>
+        <v>-4.2</v>
       </c>
       <c r="Y24" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="Z24" t="n">
-        <v>232.204</v>
+        <v>-10.9</v>
       </c>
       <c r="AA24" t="n">
-        <v>4.53</v>
+        <v>4.92</v>
       </c>
       <c r="AB24" t="n">
-        <v>-1.6</v>
+        <v>16.7</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>0.50625</v>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
@@ -2180,85 +2138,63 @@
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>reports/israel-sovereign-credit.md</t>
+          <t>reports/iraq-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Middle East (CEEMEA)</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>Ba3</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Extended Fund Facility (4-year, SDR 926.37m; Fifth Review completed Jun-26, with RSF)</t>
-        </is>
-      </c>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H25" t="n">
-        <v>2.7011</v>
+        <v>1.54</v>
       </c>
       <c r="I25" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="J25" t="n">
-        <v>3.3</v>
+        <v>1.71</v>
       </c>
       <c r="K25" t="n">
-        <v>-6.2</v>
+        <v>1.9</v>
       </c>
       <c r="L25" t="n">
-        <v>28.5</v>
+        <v>241.63</v>
       </c>
       <c r="M25" t="n">
-        <v>9.199999999999999</v>
+        <v>14.36</v>
       </c>
       <c r="P25" t="n">
-        <v>83.59999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="Q25" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="R25" t="n">
-        <v>-2.8</v>
+        <v>-5.9</v>
+      </c>
+      <c r="X25" t="n">
+        <v>2.67</v>
       </c>
       <c r="Y25" t="n">
-        <v>23</v>
+        <v>4.9</v>
       </c>
       <c r="Z25" t="n">
-        <v>21.01</v>
+        <v>232.204</v>
       </c>
       <c r="AA25" t="n">
-        <v>-3.11</v>
+        <v>4.53</v>
       </c>
       <c r="AB25" t="n">
-        <v>-6.1</v>
-      </c>
-      <c r="AC25" t="n">
-        <v>3.95</v>
+        <v>-1.6</v>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
@@ -2267,75 +2203,85 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>reports/jordan-sovereign-credit.md</t>
+          <t>reports/israel-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CIS / Central Asia</t>
+          <t>Middle East (CEEMEA)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Baa1</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
+          <t>Ba3</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Extended Fund Facility (4-year, SDR 926.37m; Fifth Review completed Jun-26, with RSF)</t>
+        </is>
+      </c>
       <c r="G26" t="n">
-        <v>4.6</v>
+        <v>2.7</v>
       </c>
       <c r="H26" t="n">
-        <v>9.24</v>
+        <v>2.7011</v>
       </c>
       <c r="I26" t="n">
-        <v>16.75</v>
+        <v>6</v>
       </c>
       <c r="J26" t="n">
-        <v>7.51</v>
+        <v>3.3</v>
       </c>
       <c r="K26" t="n">
-        <v>-1</v>
+        <v>-6.2</v>
       </c>
       <c r="L26" t="n">
-        <v>70.56999999999999</v>
+        <v>28.5</v>
       </c>
       <c r="M26" t="n">
-        <v>7.39</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P26" t="n">
-        <v>24.9</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q26" t="n">
-        <v>-1.3</v>
+        <v>-5.2</v>
+      </c>
+      <c r="R26" t="n">
+        <v>-2.8</v>
       </c>
       <c r="Y26" t="n">
-        <v>29.9</v>
+        <v>23</v>
       </c>
       <c r="Z26" t="n">
-        <v>59.792</v>
+        <v>21.01</v>
       </c>
       <c r="AA26" t="n">
-        <v>-13.41</v>
+        <v>-3.11</v>
       </c>
       <c r="AB26" t="n">
-        <v>11.5</v>
+        <v>-6.1</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>3.95</v>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
@@ -2344,76 +2290,75 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>reports/kazakhstan-sovereign-credit.md</t>
+          <t>reports/jordan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>CIS / Central Asia</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25, successor talks ongoing</t>
-        </is>
-      </c>
+          <t>Baa1</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
       <c r="G27" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="H27" t="n">
-        <v>6.76</v>
+        <v>9.24</v>
       </c>
       <c r="I27" t="n">
-        <v>8.75</v>
+        <v>16.75</v>
       </c>
       <c r="J27" t="n">
-        <v>1.99</v>
+        <v>7.51</v>
       </c>
       <c r="K27" t="n">
-        <v>-4.1</v>
+        <v>-1</v>
       </c>
       <c r="L27" t="n">
-        <v>14.702</v>
+        <v>70.56999999999999</v>
       </c>
       <c r="M27" t="n">
-        <v>4.632</v>
+        <v>7.39</v>
       </c>
       <c r="P27" t="n">
-        <v>68.5</v>
+        <v>24.9</v>
       </c>
       <c r="Q27" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="S27" t="n">
-        <v>33</v>
+        <v>-1.3</v>
       </c>
       <c r="Y27" t="n">
-        <v>34.7</v>
+        <v>29.9</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>59.792</v>
+      </c>
+      <c r="AA27" t="n">
+        <v>-13.41</v>
       </c>
       <c r="AB27" t="n">
-        <v>-2.9</v>
+        <v>11.5</v>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
@@ -2422,72 +2367,76 @@
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>reports/kenya-sovereign-credit.md</t>
+          <t>reports/kazakhstan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Middle East (GCC)</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25, successor talks ongoing</t>
+        </is>
+      </c>
       <c r="G28" t="n">
-        <v>-0.6</v>
+        <v>4.5</v>
       </c>
       <c r="H28" t="n">
-        <v>0</v>
+        <v>6.76</v>
       </c>
       <c r="I28" t="n">
-        <v>3.5</v>
+        <v>8.75</v>
       </c>
       <c r="J28" t="n">
-        <v>3.5</v>
+        <v>1.99</v>
       </c>
       <c r="K28" t="n">
-        <v>18.8</v>
+        <v>-4.1</v>
       </c>
       <c r="L28" t="n">
-        <v>32.689</v>
+        <v>14.702</v>
       </c>
       <c r="M28" t="n">
-        <v>8.4</v>
+        <v>4.632</v>
       </c>
       <c r="P28" t="n">
-        <v>2.9</v>
+        <v>68.5</v>
       </c>
       <c r="Q28" t="n">
-        <v>-18.5</v>
+        <v>-6.4</v>
+      </c>
+      <c r="S28" t="n">
+        <v>33</v>
       </c>
       <c r="Y28" t="n">
-        <v>-23.4</v>
-      </c>
-      <c r="AA28" t="n">
-        <v>32.54</v>
+        <v>34.7</v>
       </c>
       <c r="AB28" t="n">
-        <v>28.1</v>
+        <v>-2.9</v>
       </c>
       <c r="AF28" t="inlineStr">
         <is>
@@ -2496,55 +2445,72 @@
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>reports/kuwait-sovereign-credit.md</t>
+          <t>reports/kenya-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MENA</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>None; mission of 15-18 Sep-26 ended without staff-level agreement</t>
-        </is>
-      </c>
+          <t>Middle East (GCC)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="n">
-        <v>4</v>
+        <v>-0.6</v>
       </c>
       <c r="H29" t="n">
-        <v>16.66</v>
+        <v>0</v>
+      </c>
+      <c r="I29" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3.5</v>
       </c>
       <c r="K29" t="n">
-        <v>-22.5</v>
+        <v>18.8</v>
       </c>
       <c r="L29" t="n">
-        <v>38.16</v>
+        <v>32.689</v>
       </c>
       <c r="M29" t="n">
-        <v>13.6</v>
+        <v>8.4</v>
       </c>
       <c r="P29" t="n">
-        <v>139.4</v>
+        <v>2.9</v>
       </c>
       <c r="Q29" t="n">
-        <v>3.3</v>
+        <v>-18.5</v>
       </c>
       <c r="Y29" t="n">
-        <v>31.2</v>
+        <v>-23.4</v>
       </c>
       <c r="AA29" t="n">
-        <v>-9.16</v>
+        <v>32.54</v>
       </c>
       <c r="AB29" t="n">
-        <v>-4.6</v>
+        <v>28.1</v>
       </c>
       <c r="AF29" t="inlineStr">
         <is>
@@ -2553,128 +2519,120 @@
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>reports/lebanon-sovereign-credit.md</t>
+          <t>reports/kuwait-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr"/>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>None; mission of 15-18 Sep-26 ended without staff-level agreement</t>
+        </is>
+      </c>
       <c r="G30" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="H30" t="n">
-        <v>1.7817</v>
-      </c>
-      <c r="I30" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.97</v>
+        <v>16.66</v>
       </c>
       <c r="K30" t="n">
-        <v>1.4</v>
+        <v>-22.5</v>
       </c>
       <c r="L30" t="n">
-        <v>131.981</v>
+        <v>38.16</v>
       </c>
       <c r="M30" t="n">
-        <v>4.276</v>
+        <v>13.6</v>
       </c>
       <c r="P30" t="n">
-        <v>69.5</v>
+        <v>139.4</v>
       </c>
       <c r="Q30" t="n">
-        <v>-3.3</v>
-      </c>
-      <c r="X30" t="n">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
       <c r="Y30" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="Z30" t="n">
-        <v>97.798</v>
+        <v>31.2</v>
       </c>
       <c r="AA30" t="n">
-        <v>10.37</v>
+        <v>-9.16</v>
       </c>
       <c r="AB30" t="n">
-        <v>1</v>
+        <v>-4.6</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>reports/malaysia-sovereign-credit.md</t>
+          <t>reports/lebanon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Latin America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
       <c r="G31" t="n">
-        <v>1.6</v>
+        <v>4.7</v>
       </c>
       <c r="H31" t="n">
-        <v>3.2619</v>
+        <v>1.7817</v>
       </c>
       <c r="I31" t="n">
-        <v>6.5</v>
+        <v>2.75</v>
       </c>
       <c r="J31" t="n">
-        <v>3.24</v>
+        <v>0.97</v>
       </c>
       <c r="K31" t="n">
-        <v>-0.4</v>
+        <v>1.4</v>
       </c>
       <c r="L31" t="n">
-        <v>265.969</v>
+        <v>131.981</v>
       </c>
       <c r="M31" t="n">
-        <v>3.73</v>
+        <v>4.276</v>
       </c>
       <c r="P31" t="n">
-        <v>62.7</v>
+        <v>69.5</v>
       </c>
       <c r="Q31" t="n">
-        <v>-4.4</v>
+        <v>-3.3</v>
       </c>
       <c r="X31" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="Y31" t="n">
-        <v>6.8</v>
+        <v>7.5</v>
       </c>
       <c r="Z31" t="n">
-        <v>250.968</v>
+        <v>97.798</v>
       </c>
       <c r="AA31" t="n">
-        <v>-0.7</v>
+        <v>10.37</v>
       </c>
       <c r="AB31" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="AF31" t="inlineStr">
         <is>
@@ -2683,138 +2641,116 @@
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>reports/mexico-sovereign-credit.md</t>
+          <t>reports/malaysia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Montenegro</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Western Balkans (CEEMEA)</t>
+          <t>Latin America</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="H32" t="n">
-        <v>3.6043</v>
+        <v>3.2619</v>
+      </c>
+      <c r="I32" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J32" t="n">
+        <v>3.24</v>
       </c>
       <c r="K32" t="n">
-        <v>-19.4</v>
+        <v>-0.4</v>
       </c>
       <c r="L32" t="n">
-        <v>2.196</v>
+        <v>265.969</v>
       </c>
       <c r="M32" t="n">
-        <v>3.947</v>
+        <v>3.73</v>
       </c>
       <c r="P32" t="n">
-        <v>63.5</v>
+        <v>62.7</v>
       </c>
       <c r="Q32" t="n">
-        <v>-4</v>
+        <v>-4.4</v>
+      </c>
+      <c r="X32" t="n">
+        <v>1.8</v>
       </c>
       <c r="Y32" t="n">
-        <v>26.1</v>
+        <v>6.8</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>250.968</v>
       </c>
       <c r="AA32" t="n">
-        <v>-2.07</v>
+        <v>-0.7</v>
       </c>
       <c r="AB32" t="n">
-        <v>-1.6</v>
+        <v>0.3</v>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>reports/montenegro-sovereign-credit.md</t>
+          <t>reports/mexico-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>North Africa</t>
-        </is>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>Ba1</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>Flexible Credit Line (2-year, precautionary); Mid-Term Review completed Mar-26; RSF SDR 1.0bn approved Sep-23</t>
-        </is>
-      </c>
+          <t>Western Balkans (CEEMEA)</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
       <c r="H33" t="n">
-        <v>-0.3333</v>
-      </c>
-      <c r="I33" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="J33" t="n">
-        <v>2.58</v>
+        <v>3.6043</v>
       </c>
       <c r="K33" t="n">
-        <v>-3.1</v>
+        <v>-19.4</v>
       </c>
       <c r="L33" t="n">
-        <v>55.65</v>
+        <v>2.196</v>
       </c>
       <c r="M33" t="n">
-        <v>5.5</v>
+        <v>3.947</v>
       </c>
       <c r="P33" t="n">
-        <v>67.2</v>
+        <v>63.5</v>
       </c>
       <c r="Q33" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="S33" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="X33" t="n">
-        <v>-2.1</v>
+        <v>-4</v>
       </c>
       <c r="Y33" t="n">
-        <v>18</v>
-      </c>
-      <c r="Z33" t="n">
-        <v>50.756</v>
+        <v>26.1</v>
       </c>
       <c r="AA33" t="n">
-        <v>-5.83</v>
+        <v>-2.07</v>
       </c>
       <c r="AB33" t="n">
-        <v>-3.2</v>
+        <v>-1.6</v>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
@@ -2823,79 +2759,85 @@
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>reports/morocco-sovereign-credit.md</t>
+          <t>reports/montenegro-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Mozambique</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>North Africa</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>CCC (LC: SD)</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Caa3</t>
+          <t>Ba1</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>None; 2022 ECF (SDR 340.8m) lapsed Apr-25; successor arrangement under discussion after Sep-26 staff mission</t>
+          <t>Flexible Credit Line (2-year, precautionary); Mid-Term Review completed Mar-26; RSF SDR 1.0bn approved Sep-23</t>
         </is>
       </c>
       <c r="G34" t="n">
-        <v>0.5</v>
+        <v>4.9</v>
       </c>
       <c r="H34" t="n">
-        <v>6.5</v>
+        <v>-0.3333</v>
       </c>
       <c r="I34" t="n">
-        <v>9.25</v>
+        <v>2.25</v>
       </c>
       <c r="J34" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="K34" t="n">
-        <v>-43</v>
+        <v>-3.1</v>
       </c>
       <c r="L34" t="n">
-        <v>3.9</v>
+        <v>55.65</v>
       </c>
       <c r="M34" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="P34" t="n">
-        <v>94</v>
+        <v>67.2</v>
       </c>
       <c r="Q34" t="n">
-        <v>-6.5</v>
+        <v>-3.5</v>
+      </c>
+      <c r="S34" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="X34" t="n">
+        <v>-2.1</v>
       </c>
       <c r="Y34" t="n">
-        <v>4.9</v>
+        <v>18</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>50.756</v>
       </c>
       <c r="AA34" t="n">
-        <v>-2.95</v>
+        <v>-5.83</v>
       </c>
       <c r="AB34" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="AC34" t="n">
-        <v>0.9</v>
+        <v>-3.2</v>
       </c>
       <c r="AF34" t="inlineStr">
         <is>
@@ -2904,14 +2846,14 @@
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>reports/mozambique-sovereign-credit.md</t>
+          <t>reports/morocco-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Namibia</t>
+          <t>Mozambique</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -2919,39 +2861,64 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="F35" t="inlineStr"/>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>CCC (LC: SD)</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Caa3</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>None; 2022 ECF (SDR 340.8m) lapsed Apr-25; successor arrangement under discussion after Sep-26 staff mission</t>
+        </is>
+      </c>
       <c r="G35" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="H35" t="n">
-        <v>4.4106</v>
+        <v>6.5</v>
+      </c>
+      <c r="I35" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="J35" t="n">
+        <v>2.75</v>
       </c>
       <c r="K35" t="n">
-        <v>-15.7</v>
+        <v>-43</v>
       </c>
       <c r="L35" t="n">
-        <v>3.252</v>
+        <v>3.9</v>
       </c>
       <c r="M35" t="n">
-        <v>3.958</v>
+        <v>6.5</v>
       </c>
       <c r="P35" t="n">
-        <v>70.5</v>
+        <v>94</v>
       </c>
       <c r="Q35" t="n">
-        <v>-6.1</v>
+        <v>-6.5</v>
       </c>
       <c r="Y35" t="n">
-        <v>-6.3</v>
-      </c>
-      <c r="Z35" t="n">
-        <v>2.151</v>
+        <v>4.9</v>
       </c>
       <c r="AA35" t="n">
-        <v>-1.86</v>
+        <v>-2.95</v>
       </c>
       <c r="AB35" t="n">
-        <v>0.8</v>
+        <v>-0.1</v>
+      </c>
+      <c r="AC35" t="n">
+        <v>0.9</v>
       </c>
       <c r="AF35" t="inlineStr">
         <is>
@@ -2960,84 +2927,54 @@
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>reports/namibia-sovereign-credit.md</t>
+          <t>reports/mozambique-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Namibia</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>B3</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
       <c r="G36" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="H36" t="n">
-        <v>15.39</v>
-      </c>
-      <c r="I36" t="n">
-        <v>23</v>
-      </c>
-      <c r="J36" t="n">
-        <v>7.61</v>
+        <v>4.4106</v>
       </c>
       <c r="K36" t="n">
-        <v>5.8</v>
+        <v>-15.7</v>
       </c>
       <c r="L36" t="n">
-        <v>54.98</v>
+        <v>3.252</v>
       </c>
       <c r="M36" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="O36" t="n">
-        <v>14.4</v>
+        <v>3.958</v>
       </c>
       <c r="P36" t="n">
-        <v>32.3</v>
+        <v>70.5</v>
       </c>
       <c r="Q36" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="S36" t="n">
-        <v>55</v>
-      </c>
-      <c r="X36" t="n">
-        <v>-0.51</v>
+        <v>-6.1</v>
       </c>
       <c r="Y36" t="n">
-        <v>30.8</v>
+        <v>-6.3</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>2.151</v>
       </c>
       <c r="AA36" t="n">
-        <v>15.61</v>
+        <v>-1.86</v>
       </c>
       <c r="AB36" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="AC36" t="n">
-        <v>15.12</v>
+        <v>0.8</v>
       </c>
       <c r="AF36" t="inlineStr">
         <is>
@@ -3046,80 +2983,84 @@
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>reports/nigeria-sovereign-credit.md</t>
+          <t>reports/namibia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CEEMEA - Western Balkans</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>PLL concluded Nov-24</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="H37" t="n">
-        <v>2.5729</v>
+        <v>15.39</v>
       </c>
       <c r="I37" t="n">
-        <v>4.25</v>
+        <v>23</v>
       </c>
       <c r="J37" t="n">
-        <v>1.68</v>
+        <v>7.61</v>
       </c>
       <c r="K37" t="n">
-        <v>-5</v>
+        <v>5.8</v>
       </c>
       <c r="L37" t="n">
-        <v>5.51</v>
+        <v>54.98</v>
       </c>
       <c r="M37" t="n">
-        <v>4.2</v>
+        <v>9.199999999999999</v>
+      </c>
+      <c r="O37" t="n">
+        <v>14.4</v>
       </c>
       <c r="P37" t="n">
-        <v>55.2</v>
+        <v>32.3</v>
       </c>
       <c r="Q37" t="n">
-        <v>-4.2</v>
+        <v>-4.4</v>
+      </c>
+      <c r="S37" t="n">
+        <v>55</v>
       </c>
       <c r="X37" t="n">
-        <v>1.52</v>
+        <v>-0.51</v>
       </c>
       <c r="Y37" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="Z37" t="n">
-        <v>4.474</v>
+        <v>30.8</v>
       </c>
       <c r="AA37" t="n">
-        <v>-0.99</v>
+        <v>15.61</v>
       </c>
       <c r="AB37" t="n">
-        <v>-2.6</v>
+        <v>4.6</v>
       </c>
       <c r="AC37" t="n">
-        <v>2.16</v>
+        <v>15.12</v>
       </c>
       <c r="AF37" t="inlineStr">
         <is>
@@ -3128,67 +3069,80 @@
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>reports/north-macedonia-sovereign-credit.md</t>
+          <t>reports/nigeria-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Middle East (GCC)</t>
+          <t>CEEMEA - Western Balkans</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>Baa3</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>PLL concluded Nov-24</t>
         </is>
       </c>
       <c r="G38" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="H38" t="n">
-        <v>3.3771</v>
+        <v>2.5729</v>
+      </c>
+      <c r="I38" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1.68</v>
       </c>
       <c r="K38" t="n">
-        <v>2.5</v>
+        <v>-5</v>
       </c>
       <c r="L38" t="n">
-        <v>18.38</v>
+        <v>5.51</v>
       </c>
       <c r="M38" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="P38" t="n">
-        <v>34.7</v>
+        <v>55.2</v>
       </c>
       <c r="Q38" t="n">
-        <v>0.6</v>
+        <v>-4.2</v>
+      </c>
+      <c r="X38" t="n">
+        <v>1.52</v>
       </c>
       <c r="Y38" t="n">
-        <v>9.199999999999999</v>
+        <v>7.2</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>4.474</v>
+      </c>
+      <c r="AA38" t="n">
+        <v>-0.99</v>
       </c>
       <c r="AB38" t="n">
-        <v>15.6</v>
+        <v>-2.6</v>
+      </c>
+      <c r="AC38" t="n">
+        <v>2.16</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -3197,54 +3151,67 @@
       </c>
       <c r="AG38" t="inlineStr">
         <is>
-          <t>reports/oman-sovereign-credit.md</t>
+          <t>reports/north-macedonia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>South Asia</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr"/>
+          <t>Middle East (GCC)</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Baa3</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
       <c r="G39" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
       <c r="H39" t="n">
-        <v>10.2591</v>
+        <v>3.3771</v>
       </c>
       <c r="K39" t="n">
-        <v>-0.4</v>
+        <v>2.5</v>
       </c>
       <c r="L39" t="n">
-        <v>27.993</v>
+        <v>18.38</v>
       </c>
       <c r="M39" t="n">
-        <v>3.755</v>
+        <v>5</v>
       </c>
       <c r="P39" t="n">
-        <v>70.09999999999999</v>
+        <v>34.7</v>
       </c>
       <c r="Q39" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="X39" t="n">
-        <v>1.02</v>
+        <v>0.6</v>
       </c>
       <c r="Y39" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="AA39" t="n">
-        <v>-0.14</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AB39" t="n">
-        <v>-2.3</v>
+        <v>15.6</v>
       </c>
       <c r="AF39" t="inlineStr">
         <is>
@@ -3253,128 +3220,119 @@
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>reports/pakistan-sovereign-credit.md</t>
+          <t>reports/oman-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Latin America</t>
+          <t>South Asia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
       <c r="G40" t="n">
-        <v>2.8</v>
+        <v>3.6</v>
       </c>
       <c r="H40" t="n">
-        <v>4.0636</v>
-      </c>
-      <c r="I40" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="J40" t="n">
-        <v>0.19</v>
+        <v>10.2591</v>
       </c>
       <c r="K40" t="n">
-        <v>3.4</v>
+        <v>-0.4</v>
       </c>
       <c r="L40" t="n">
-        <v>95.26900000000001</v>
+        <v>27.993</v>
       </c>
       <c r="M40" t="n">
-        <v>10.423</v>
+        <v>3.755</v>
       </c>
       <c r="P40" t="n">
-        <v>30</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="Q40" t="n">
-        <v>-2</v>
+        <v>-3.2</v>
       </c>
       <c r="X40" t="n">
-        <v>1.8</v>
+        <v>1.02</v>
       </c>
       <c r="Y40" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="Z40" t="n">
-        <v>87.288</v>
+        <v>22.8</v>
       </c>
       <c r="AA40" t="n">
-        <v>12.01</v>
+        <v>-0.14</v>
       </c>
       <c r="AB40" t="n">
-        <v>2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="AF40" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>reports/peru-sovereign-credit.md</t>
+          <t>reports/pakistan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Latin America</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
-        <v>4.1</v>
+        <v>2.8</v>
       </c>
       <c r="H41" t="n">
-        <v>6.3629</v>
+        <v>4.0636</v>
       </c>
       <c r="I41" t="n">
-        <v>5</v>
+        <v>4.25</v>
       </c>
       <c r="J41" t="n">
-        <v>-1.36</v>
+        <v>0.19</v>
       </c>
       <c r="K41" t="n">
-        <v>-4.4</v>
+        <v>3.4</v>
       </c>
       <c r="L41" t="n">
-        <v>103.316</v>
+        <v>95.26900000000001</v>
       </c>
       <c r="M41" t="n">
-        <v>7.306</v>
+        <v>10.423</v>
       </c>
       <c r="P41" t="n">
-        <v>60.2</v>
+        <v>30</v>
       </c>
       <c r="Q41" t="n">
-        <v>-3.7</v>
+        <v>-2</v>
       </c>
       <c r="X41" t="n">
-        <v>-0.19</v>
+        <v>1.8</v>
       </c>
       <c r="Y41" t="n">
-        <v>-2</v>
+        <v>16.3</v>
       </c>
       <c r="Z41" t="n">
-        <v>93.018</v>
+        <v>87.288</v>
       </c>
       <c r="AA41" t="n">
-        <v>-22.11</v>
+        <v>12.01</v>
       </c>
       <c r="AB41" t="n">
-        <v>-1.4</v>
+        <v>2.5</v>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
@@ -3383,63 +3341,63 @@
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>reports/philippines-sovereign-credit.md</t>
+          <t>reports/peru-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Central Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
-        <v>3.3</v>
+        <v>4.1</v>
       </c>
       <c r="H42" t="n">
-        <v>3.2123</v>
+        <v>6.3629</v>
       </c>
       <c r="I42" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="J42" t="n">
-        <v>0.54</v>
+        <v>-1.36</v>
       </c>
       <c r="K42" t="n">
-        <v>-1.1</v>
+        <v>-4.4</v>
       </c>
       <c r="L42" t="n">
-        <v>304.971</v>
+        <v>103.316</v>
       </c>
       <c r="M42" t="n">
-        <v>5.861</v>
+        <v>7.306</v>
       </c>
       <c r="P42" t="n">
-        <v>65.7</v>
+        <v>60.2</v>
       </c>
       <c r="Q42" t="n">
-        <v>-6.7</v>
+        <v>-3.7</v>
       </c>
       <c r="X42" t="n">
-        <v>1.5</v>
+        <v>-0.19</v>
       </c>
       <c r="Y42" t="n">
-        <v>16.9</v>
+        <v>-2</v>
       </c>
       <c r="Z42" t="n">
-        <v>277.21</v>
+        <v>93.018</v>
       </c>
       <c r="AA42" t="n">
-        <v>-13.87</v>
+        <v>-22.11</v>
       </c>
       <c r="AB42" t="n">
-        <v>-1.1</v>
+        <v>-1.4</v>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
@@ -3448,279 +3406,279 @@
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>reports/poland-sovereign-credit.md</t>
+          <t>reports/philippines-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>GCC</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>AA</t>
+          <t>Central Europe</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
-        <v>-8.6</v>
+        <v>3.3</v>
       </c>
       <c r="H43" t="n">
-        <v>0.73</v>
+        <v>3.2123</v>
       </c>
       <c r="I43" t="n">
-        <v>4.35</v>
+        <v>3.75</v>
       </c>
       <c r="J43" t="n">
-        <v>3.62</v>
+        <v>0.54</v>
       </c>
       <c r="K43" t="n">
-        <v>11</v>
+        <v>-1.1</v>
       </c>
       <c r="L43" t="n">
-        <v>61.1</v>
+        <v>304.971</v>
       </c>
       <c r="M43" t="n">
-        <v>7.45</v>
+        <v>5.861</v>
       </c>
       <c r="P43" t="n">
-        <v>43.3</v>
+        <v>65.7</v>
       </c>
       <c r="Q43" t="n">
-        <v>-3.4</v>
+        <v>-6.7</v>
+      </c>
+      <c r="X43" t="n">
+        <v>1.5</v>
       </c>
       <c r="Y43" t="n">
-        <v>10.4</v>
+        <v>16.9</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>277.21</v>
       </c>
       <c r="AA43" t="n">
-        <v>28.52</v>
+        <v>-13.87</v>
       </c>
       <c r="AB43" t="n">
-        <v>14.7</v>
+        <v>-1.1</v>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>reports/qatar-sovereign-credit.md</t>
+          <t>reports/poland-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Central Europe</t>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>AA</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
-        <v>0.7</v>
+        <v>-8.6</v>
       </c>
       <c r="H44" t="n">
-        <v>8.16</v>
+        <v>0.73</v>
       </c>
       <c r="I44" t="n">
-        <v>6.5</v>
+        <v>4.35</v>
       </c>
       <c r="J44" t="n">
-        <v>-1.66</v>
+        <v>3.62</v>
       </c>
       <c r="K44" t="n">
-        <v>-6.8</v>
+        <v>11</v>
       </c>
       <c r="L44" t="n">
-        <v>90.04300000000001</v>
+        <v>61.1</v>
       </c>
       <c r="M44" t="n">
-        <v>5.528</v>
+        <v>7.45</v>
       </c>
       <c r="P44" t="n">
-        <v>61.9</v>
+        <v>43.3</v>
       </c>
       <c r="Q44" t="n">
-        <v>-6.2</v>
-      </c>
-      <c r="X44" t="n">
-        <v>1.95</v>
+        <v>-3.4</v>
       </c>
       <c r="Y44" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="Z44" t="n">
-        <v>72.172</v>
+        <v>10.4</v>
       </c>
       <c r="AA44" t="n">
-        <v>-32.2</v>
+        <v>28.52</v>
       </c>
       <c r="AB44" t="n">
-        <v>-0.5</v>
+        <v>14.7</v>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>reports/romania-sovereign-credit.md</t>
+          <t>reports/qatar-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>38-month ECF (reported)</t>
-        </is>
-      </c>
+          <t>Central Europe</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>9.699999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="H45" t="n">
-        <v>15.7</v>
+        <v>8.16</v>
       </c>
       <c r="I45" t="n">
-        <v>8.75</v>
+        <v>6.5</v>
       </c>
       <c r="J45" t="n">
-        <v>-6.95</v>
+        <v>-1.66</v>
       </c>
       <c r="K45" t="n">
-        <v>-15</v>
+        <v>-6.8</v>
       </c>
       <c r="L45" t="n">
-        <v>2.2</v>
+        <v>90.04300000000001</v>
       </c>
       <c r="M45" t="n">
-        <v>4</v>
-      </c>
-      <c r="O45" t="n">
-        <v>63</v>
+        <v>5.528</v>
       </c>
       <c r="P45" t="n">
-        <v>77.5</v>
+        <v>61.9</v>
       </c>
       <c r="Q45" t="n">
-        <v>-4.8</v>
+        <v>-6.2</v>
+      </c>
+      <c r="X45" t="n">
+        <v>1.95</v>
       </c>
       <c r="Y45" t="n">
-        <v>-16.4</v>
+        <v>2.9</v>
       </c>
       <c r="Z45" t="n">
-        <v>1.795</v>
+        <v>72.172</v>
       </c>
       <c r="AA45" t="n">
-        <v>-1.98</v>
+        <v>-32.2</v>
       </c>
       <c r="AB45" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AC45" t="n">
-        <v>0.62</v>
+        <v>-0.5</v>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>reports/rwanda-sovereign-credit.md</t>
+          <t>reports/romania-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Middle East</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr"/>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>38-month ECF (reported)</t>
+        </is>
+      </c>
       <c r="G46" t="n">
-        <v>3.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H46" t="n">
-        <v>1.82</v>
+        <v>15.7</v>
       </c>
       <c r="I46" t="n">
-        <v>4.5</v>
+        <v>8.75</v>
       </c>
       <c r="J46" t="n">
-        <v>2.68</v>
+        <v>-6.95</v>
       </c>
       <c r="K46" t="n">
-        <v>-1.6</v>
+        <v>-15</v>
       </c>
       <c r="L46" t="n">
-        <v>488.684</v>
+        <v>2.2</v>
       </c>
       <c r="M46" t="n">
-        <v>15.6</v>
+        <v>4</v>
+      </c>
+      <c r="O46" t="n">
+        <v>63</v>
       </c>
       <c r="P46" t="n">
-        <v>32.1</v>
+        <v>77.5</v>
       </c>
       <c r="Q46" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="X46" t="n">
-        <v>-0.31</v>
+        <v>-4.8</v>
       </c>
       <c r="Y46" t="n">
-        <v>10</v>
+        <v>-16.4</v>
       </c>
       <c r="Z46" t="n">
-        <v>482.147</v>
+        <v>1.795</v>
       </c>
       <c r="AA46" t="n">
-        <v>-25.78</v>
+        <v>-1.98</v>
       </c>
       <c r="AB46" t="n">
-        <v>15.9</v>
+        <v>-0</v>
+      </c>
+      <c r="AC46" t="n">
+        <v>0.62</v>
       </c>
       <c r="AF46" t="inlineStr">
         <is>
@@ -3729,62 +3687,63 @@
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>reports/saudi-arabia-sovereign-credit.md</t>
+          <t>reports/rwanda-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa (WAEMU)</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Caa2</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Staff-level agreement on new arrangement replacing suspended USD 1.8B facility; Board consideration 15-Dec-26</t>
-        </is>
-      </c>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr"/>
       <c r="G47" t="n">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
       <c r="H47" t="n">
-        <v>1.2</v>
+        <v>1.82</v>
       </c>
       <c r="I47" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="J47" t="n">
-        <v>1.8</v>
+        <v>2.68</v>
       </c>
       <c r="K47" t="n">
-        <v>-6.2</v>
+        <v>-1.6</v>
+      </c>
+      <c r="L47" t="n">
+        <v>488.684</v>
+      </c>
+      <c r="M47" t="n">
+        <v>15.6</v>
       </c>
       <c r="P47" t="n">
-        <v>132</v>
+        <v>32.1</v>
       </c>
       <c r="Q47" t="n">
-        <v>-6.7</v>
+        <v>-3.5</v>
+      </c>
+      <c r="X47" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>482.147</v>
+      </c>
+      <c r="AA47" t="n">
+        <v>-25.78</v>
       </c>
       <c r="AB47" t="n">
-        <v>-2.4</v>
-      </c>
-      <c r="AC47" t="n">
-        <v>3.2</v>
+        <v>15.9</v>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
@@ -3793,82 +3752,62 @@
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/saudi-arabia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CEEMEA - Western Balkans</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Sub-Saharan Africa (WAEMU)</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Policy Coordination Instrument (36-month, non-financing)</t>
+          <t>Staff-level agreement on new arrangement replacing suspended USD 1.8B facility; Board consideration 15-Dec-26</t>
         </is>
       </c>
       <c r="G48" t="n">
-        <v>3.8</v>
+        <v>6.8</v>
       </c>
       <c r="H48" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I48" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J48" t="n">
-        <v>3.55</v>
+        <v>1.8</v>
       </c>
       <c r="K48" t="n">
-        <v>-4.1</v>
-      </c>
-      <c r="L48" t="n">
-        <v>35.71</v>
-      </c>
-      <c r="M48" t="n">
-        <v>6.2</v>
+        <v>-6.2</v>
       </c>
       <c r="P48" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="Q48" t="n">
-        <v>-3.25</v>
-      </c>
-      <c r="X48" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="Y48" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z48" t="n">
-        <v>30.033</v>
-      </c>
-      <c r="AA48" t="n">
-        <v>-4.36</v>
+        <v>-6.7</v>
       </c>
       <c r="AB48" t="n">
-        <v>-1.4</v>
+        <v>-2.4</v>
+      </c>
+      <c r="AC48" t="n">
+        <v>3.2</v>
       </c>
       <c r="AF48" t="inlineStr">
         <is>
@@ -3877,29 +3816,29 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>CEEMEA - Western Balkans</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -3909,53 +3848,50 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>Policy Coordination Instrument (36-month, non-financing)</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="H49" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I49" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J49" t="n">
-        <v>2.9</v>
+        <v>3.55</v>
       </c>
       <c r="K49" t="n">
-        <v>-1.6</v>
+        <v>-4.1</v>
       </c>
       <c r="L49" t="n">
-        <v>75.95999999999999</v>
+        <v>35.71</v>
       </c>
       <c r="M49" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="P49" t="n">
-        <v>77.2</v>
+        <v>43.3</v>
       </c>
       <c r="Q49" t="n">
-        <v>-3.8</v>
-      </c>
-      <c r="S49" t="n">
-        <v>20</v>
+        <v>-3.25</v>
       </c>
       <c r="X49" t="n">
-        <v>1.23</v>
+        <v>1.37</v>
       </c>
       <c r="Y49" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="Z49" t="n">
-        <v>74.307</v>
+        <v>30.033</v>
       </c>
       <c r="AA49" t="n">
-        <v>-1.32</v>
+        <v>-4.36</v>
       </c>
       <c r="AB49" t="n">
-        <v>-0.9</v>
+        <v>-1.4</v>
       </c>
       <c r="AF49" t="inlineStr">
         <is>
@@ -3964,51 +3900,85 @@
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Central Asia</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr"/>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
       <c r="G50" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H50" t="n">
-        <v>4.0609</v>
+        <v>4.4</v>
+      </c>
+      <c r="I50" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="J50" t="n">
+        <v>2.9</v>
       </c>
       <c r="K50" t="n">
-        <v>6.3</v>
+        <v>-1.6</v>
       </c>
       <c r="L50" t="n">
-        <v>6.395</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="M50" t="n">
-        <v>5.749</v>
+        <v>5.8</v>
       </c>
       <c r="P50" t="n">
-        <v>21.9</v>
+        <v>77.2</v>
       </c>
       <c r="Q50" t="n">
-        <v>-2.5</v>
+        <v>-3.8</v>
+      </c>
+      <c r="S50" t="n">
+        <v>20</v>
+      </c>
+      <c r="X50" t="n">
+        <v>1.23</v>
       </c>
       <c r="Y50" t="n">
-        <v>45.9</v>
+        <v>7.8</v>
+      </c>
+      <c r="Z50" t="n">
+        <v>74.307</v>
       </c>
       <c r="AA50" t="n">
-        <v>3.48</v>
+        <v>-1.32</v>
       </c>
       <c r="AB50" t="n">
-        <v>-0.8</v>
+        <v>-0.9</v>
       </c>
       <c r="AF50" t="inlineStr">
         <is>
@@ -4017,228 +3987,195 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>reports/tajikistan-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Central Asia</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="H51" t="n">
-        <v>2.5265</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" t="n">
-        <v>-1.53</v>
+        <v>4.0609</v>
       </c>
       <c r="K51" t="n">
-        <v>0.7</v>
+        <v>6.3</v>
       </c>
       <c r="L51" t="n">
-        <v>283.137</v>
+        <v>6.395</v>
       </c>
       <c r="M51" t="n">
-        <v>8.051</v>
+        <v>5.749</v>
       </c>
       <c r="P51" t="n">
-        <v>66.8</v>
+        <v>21.9</v>
       </c>
       <c r="Q51" t="n">
-        <v>-2.2</v>
-      </c>
-      <c r="X51" t="n">
-        <v>0.21</v>
+        <v>-2.5</v>
       </c>
       <c r="Y51" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="Z51" t="n">
-        <v>302.852</v>
+        <v>45.9</v>
       </c>
       <c r="AA51" t="n">
-        <v>8.08</v>
+        <v>3.48</v>
       </c>
       <c r="AB51" t="n">
-        <v>-3.9</v>
+        <v>-0.8</v>
       </c>
       <c r="AF51" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>reports/thailand-sovereign-credit.md</t>
+          <t>reports/tajikistan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>North Africa</t>
-        </is>
-      </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>$1.9bn Extended Fund Facility agreed at staff level Oct-22; never approved by the Executive Board; frozen</t>
-        </is>
-      </c>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="H52" t="n">
-        <v>5.6</v>
+        <v>2.5265</v>
       </c>
       <c r="I52" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J52" t="n">
-        <v>1.4</v>
+        <v>-1.53</v>
       </c>
       <c r="K52" t="n">
-        <v>-4.2</v>
+        <v>0.7</v>
       </c>
       <c r="L52" t="n">
-        <v>9.079000000000001</v>
+        <v>283.137</v>
       </c>
       <c r="M52" t="n">
-        <v>3</v>
+        <v>8.051</v>
       </c>
       <c r="P52" t="n">
-        <v>82</v>
+        <v>66.8</v>
       </c>
       <c r="Q52" t="n">
-        <v>-5.2</v>
+        <v>-2.2</v>
       </c>
       <c r="X52" t="n">
-        <v>1.63</v>
+        <v>0.21</v>
       </c>
       <c r="Y52" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>302.852</v>
       </c>
       <c r="AA52" t="n">
-        <v>-1.33</v>
+        <v>8.08</v>
       </c>
       <c r="AB52" t="n">
-        <v>-1.2</v>
-      </c>
-      <c r="AC52" t="n">
-        <v>0.15</v>
+        <v>-3.9</v>
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>reports/tunisia-sovereign-credit.md</t>
+          <t>reports/thailand-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CEEMEA</t>
+          <t>North Africa</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Ba3</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr"/>
+          <t>Caa1</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>$1.9bn Extended Fund Facility agreed at staff level Oct-22; never approved by the Executive Board; frozen</t>
+        </is>
+      </c>
       <c r="G53" t="n">
-        <v>3.4</v>
+        <v>2.1</v>
       </c>
       <c r="H53" t="n">
-        <v>29.73</v>
+        <v>5.6</v>
       </c>
       <c r="I53" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="J53" t="n">
-        <v>12.5</v>
+        <v>1.4</v>
       </c>
       <c r="K53" t="n">
-        <v>-2.7</v>
+        <v>-4.2</v>
       </c>
       <c r="L53" t="n">
-        <v>174.4</v>
+        <v>9.079000000000001</v>
       </c>
       <c r="M53" t="n">
-        <v>5.128</v>
-      </c>
-      <c r="N53" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="O53" t="n">
-        <v>31.8</v>
+        <v>3</v>
       </c>
       <c r="P53" t="n">
-        <v>29.5</v>
+        <v>82</v>
       </c>
       <c r="Q53" t="n">
         <v>-5.2</v>
       </c>
       <c r="X53" t="n">
-        <v>0.31</v>
+        <v>1.63</v>
       </c>
       <c r="Y53" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="Z53" t="n">
-        <v>137.109</v>
+        <v>6.8</v>
       </c>
       <c r="AA53" t="n">
-        <v>-38.89</v>
+        <v>-1.33</v>
       </c>
       <c r="AB53" t="n">
-        <v>-1</v>
+        <v>-1.2</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>0.15</v>
       </c>
       <c r="AF53" t="inlineStr">
         <is>
@@ -4247,14 +4184,14 @@
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/tunisia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4264,65 +4201,67 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>4-year EFF (first review completed 20-Jul-26, SDR 503M, about $690M disbursed)</t>
-        </is>
-      </c>
+          <t>Ba3</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr"/>
       <c r="G54" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="H54" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I54" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J54" t="n">
-        <v>7.9</v>
+        <v>12.5</v>
       </c>
       <c r="K54" t="n">
-        <v>-18.9</v>
+        <v>-2.7</v>
       </c>
       <c r="L54" t="n">
-        <v>47.1</v>
+        <v>174.4</v>
       </c>
       <c r="M54" t="n">
-        <v>5.6</v>
+        <v>5.128</v>
+      </c>
+      <c r="N54" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="O54" t="n">
+        <v>31.8</v>
       </c>
       <c r="P54" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
       </c>
       <c r="Q54" t="n">
-        <v>-18.4</v>
+        <v>-5.2</v>
       </c>
       <c r="X54" t="n">
-        <v>-0.5</v>
+        <v>0.31</v>
       </c>
       <c r="Y54" t="n">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="Z54" t="n">
-        <v>38.646</v>
+        <v>137.109</v>
       </c>
       <c r="AA54" t="n">
-        <v>-24.81</v>
+        <v>-38.89</v>
       </c>
       <c r="AB54" t="n">
-        <v>-2.3</v>
+        <v>-1</v>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
@@ -4331,61 +4270,82 @@
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MENA / GCC</t>
+          <t>CEEMEA</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr"/>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>4-year EFF (first review completed 20-Jul-26, SDR 503M, about $690M disbursed)</t>
+        </is>
+      </c>
       <c r="G55" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="H55" t="n">
-        <v>2.05</v>
+        <v>8.1</v>
+      </c>
+      <c r="I55" t="n">
+        <v>16</v>
+      </c>
+      <c r="J55" t="n">
+        <v>7.9</v>
       </c>
       <c r="K55" t="n">
-        <v>11.4</v>
+        <v>-18.9</v>
       </c>
       <c r="L55" t="n">
-        <v>259.7</v>
+        <v>47.1</v>
       </c>
       <c r="M55" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="P55" t="n">
-        <v>31.4</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="Q55" t="n">
-        <v>4.9</v>
+        <v>-18.4</v>
       </c>
       <c r="X55" t="n">
-        <v>-1.12</v>
+        <v>-0.5</v>
       </c>
       <c r="Y55" t="n">
-        <v>-3.1</v>
+        <v>5.7</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>38.646</v>
+      </c>
+      <c r="AA55" t="n">
+        <v>-24.81</v>
       </c>
       <c r="AB55" t="n">
-        <v>13.2</v>
+        <v>-2.3</v>
       </c>
       <c r="AF55" t="inlineStr">
         <is>
@@ -4394,73 +4354,61 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>reports/uae-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Central Asia / CIS</t>
+          <t>MENA / GCC</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AA-</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Ba2</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>None (Article IV surveillance only)</t>
-        </is>
-      </c>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr"/>
       <c r="G56" t="n">
-        <v>8.699999999999999</v>
+        <v>3.1</v>
       </c>
       <c r="H56" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="I56" t="n">
-        <v>14</v>
-      </c>
-      <c r="J56" t="n">
-        <v>7.8</v>
+        <v>2.05</v>
       </c>
       <c r="K56" t="n">
-        <v>-1.3</v>
+        <v>11.4</v>
       </c>
       <c r="L56" t="n">
-        <v>72.13</v>
+        <v>259.7</v>
       </c>
       <c r="M56" t="n">
-        <v>12</v>
+        <v>5.2</v>
       </c>
       <c r="P56" t="n">
-        <v>27</v>
+        <v>31.4</v>
       </c>
       <c r="Q56" t="n">
-        <v>-2.1</v>
+        <v>4.9</v>
+      </c>
+      <c r="X56" t="n">
+        <v>-1.12</v>
       </c>
       <c r="Y56" t="n">
-        <v>32</v>
-      </c>
-      <c r="AA56" t="n">
-        <v>-11.23</v>
+        <v>-3.1</v>
+      </c>
+      <c r="AB56" t="n">
+        <v>13.2</v>
       </c>
       <c r="AF56" t="inlineStr">
         <is>
@@ -4469,89 +4417,164 @@
       </c>
       <c r="AG56" t="inlineStr">
         <is>
-          <t>reports/uzbekistan-sovereign-credit.md</t>
+          <t>reports/uae-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Central Asia / CIS</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>None (Article IV surveillance only)</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H57" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I57" t="n">
+        <v>14</v>
+      </c>
+      <c r="J57" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="K57" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="L57" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="M57" t="n">
+        <v>12</v>
+      </c>
+      <c r="P57" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>32</v>
+      </c>
+      <c r="AA57" t="n">
+        <v>-11.23</v>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>09-Oct-26</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>reports/uzbekistan-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B58" t="inlineStr">
         <is>
           <t>Sub-Saharan Africa</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C58" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D58" t="inlineStr">
         <is>
           <t>CCC+</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E58" t="inlineStr">
         <is>
           <t>Caa2</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F58" t="inlineStr">
         <is>
           <t>38-month ECF completed Jan-26 (sixth and final review); successor programme under negotiation</t>
         </is>
       </c>
-      <c r="G57" t="n">
+      <c r="G58" t="n">
         <v>4.3</v>
       </c>
-      <c r="H57" t="n">
+      <c r="H58" t="n">
         <v>6.1</v>
       </c>
-      <c r="I57" t="n">
+      <c r="I58" t="n">
         <v>10.75</v>
       </c>
-      <c r="J57" t="n">
+      <c r="J58" t="n">
         <v>4.65</v>
       </c>
-      <c r="K57" t="n">
+      <c r="K58" t="n">
         <v>0.9</v>
       </c>
-      <c r="L57" t="n">
+      <c r="L58" t="n">
         <v>5.8</v>
       </c>
-      <c r="M57" t="n">
+      <c r="M58" t="n">
         <v>4.2</v>
       </c>
-      <c r="P57" t="n">
+      <c r="P58" t="n">
         <v>91</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="Q58" t="n">
         <v>-4.9</v>
       </c>
-      <c r="S57" t="n">
+      <c r="S58" t="n">
         <v>35</v>
       </c>
-      <c r="X57" t="n">
+      <c r="X58" t="n">
         <v>2.27</v>
       </c>
-      <c r="Y57" t="n">
+      <c r="Y58" t="n">
         <v>25.6</v>
       </c>
-      <c r="AA57" t="n">
+      <c r="AA58" t="n">
         <v>-0.9</v>
       </c>
-      <c r="AB57" t="n">
+      <c r="AB58" t="n">
         <v>5.1</v>
       </c>
-      <c r="AF57" t="inlineStr">
+      <c r="AF58" t="inlineStr">
         <is>
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="AG57" t="inlineStr">
+      <c r="AG58" t="inlineStr">
         <is>
           <t>reports/zambia-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-09 08:42
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG58"/>
+  <dimension ref="A1:AG59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1875,121 +1875,79 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Gulf support and anchors for EM sovereigns</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Central Europe</t>
+          <t>Thematic: Gulf (GCC) support for EM sovereigns (Pakistan, Egypt, Bahrain)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
-      <c r="G21" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="H21" t="n">
-        <v>1.2826</v>
-      </c>
-      <c r="I21" t="n">
-        <v>5.5</v>
-      </c>
-      <c r="J21" t="n">
-        <v>4.22</v>
-      </c>
-      <c r="K21" t="n">
-        <v>-0.4</v>
-      </c>
-      <c r="L21" t="n">
-        <v>73.621</v>
-      </c>
-      <c r="M21" t="n">
-        <v>3.495</v>
-      </c>
-      <c r="P21" t="n">
-        <v>77.90000000000001</v>
-      </c>
-      <c r="Q21" t="n">
-        <v>-5.5</v>
-      </c>
-      <c r="X21" t="n">
-        <v>2.27</v>
-      </c>
-      <c r="Y21" t="n">
-        <v>30.3</v>
-      </c>
-      <c r="Z21" t="n">
-        <v>66.95</v>
-      </c>
-      <c r="AA21" t="n">
-        <v>2.37</v>
-      </c>
-      <c r="AB21" t="n">
-        <v>-1.1</v>
-      </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>reports/hungary-sovereign-credit.md</t>
+          <t>reports/gulf-support-and-anchors-for-em-s-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Central Europe</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="n">
-        <v>6.5</v>
+        <v>1.7</v>
       </c>
       <c r="H22" t="n">
-        <v>4.4412</v>
+        <v>1.2826</v>
       </c>
       <c r="I22" t="n">
-        <v>5.25</v>
+        <v>5.5</v>
       </c>
       <c r="J22" t="n">
-        <v>0.8100000000000001</v>
+        <v>4.22</v>
       </c>
       <c r="K22" t="n">
-        <v>-2</v>
+        <v>-0.4</v>
       </c>
       <c r="L22" t="n">
-        <v>751.764</v>
+        <v>73.621</v>
       </c>
       <c r="M22" t="n">
-        <v>7.851</v>
+        <v>3.495</v>
       </c>
       <c r="P22" t="n">
-        <v>83.40000000000001</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="Q22" t="n">
-        <v>-7.4</v>
+        <v>-5.5</v>
       </c>
       <c r="X22" t="n">
-        <v>-2.75</v>
+        <v>2.27</v>
       </c>
       <c r="Y22" t="n">
-        <v>8.1</v>
+        <v>30.3</v>
       </c>
       <c r="Z22" t="n">
-        <v>715.745</v>
+        <v>66.95</v>
       </c>
       <c r="AA22" t="n">
-        <v>-28.25</v>
+        <v>2.37</v>
       </c>
       <c r="AB22" t="n">
-        <v>-2.8</v>
+        <v>-1.1</v>
       </c>
       <c r="AF22" t="inlineStr">
         <is>
@@ -1998,14 +1956,14 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>reports/india-sovereign-credit.md</t>
+          <t>reports/hungary-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2015,47 +1973,47 @@
       </c>
       <c r="F23" t="inlineStr"/>
       <c r="G23" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="H23" t="n">
-        <v>2.8821</v>
+        <v>4.4412</v>
       </c>
       <c r="I23" t="n">
-        <v>5.75</v>
+        <v>5.25</v>
       </c>
       <c r="J23" t="n">
-        <v>2.87</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="K23" t="n">
-        <v>-1.1</v>
+        <v>-2</v>
       </c>
       <c r="L23" t="n">
-        <v>146.492</v>
+        <v>751.764</v>
       </c>
       <c r="M23" t="n">
-        <v>5.514</v>
+        <v>7.851</v>
       </c>
       <c r="P23" t="n">
-        <v>41.5</v>
+        <v>83.40000000000001</v>
       </c>
       <c r="Q23" t="n">
-        <v>-2.9</v>
+        <v>-7.4</v>
       </c>
       <c r="X23" t="n">
-        <v>-3.03</v>
+        <v>-2.75</v>
       </c>
       <c r="Y23" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>715.745</v>
+      </c>
+      <c r="AA23" t="n">
+        <v>-28.25</v>
+      </c>
+      <c r="AB23" t="n">
         <v>-2.8</v>
       </c>
-      <c r="Z23" t="n">
-        <v>75.541</v>
-      </c>
-      <c r="AA23" t="n">
-        <v>-14.36</v>
-      </c>
-      <c r="AB23" t="n">
-        <v>0.4</v>
-      </c>
       <c r="AF23" t="inlineStr">
         <is>
           <t>08-Oct-26</t>
@@ -2063,138 +2021,138 @@
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>reports/indonesia-sovereign-credit.md</t>
+          <t>reports/india-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MENA</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>None active (Article IV surveillance and Post-Financing Assessment; last SBA expired 2018)</t>
-        </is>
-      </c>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
       <c r="G24" t="n">
-        <v>-6.8</v>
+        <v>5</v>
       </c>
       <c r="H24" t="n">
-        <v>3.0928</v>
+        <v>2.8821</v>
+      </c>
+      <c r="I24" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2.87</v>
       </c>
       <c r="K24" t="n">
-        <v>-5.3</v>
+        <v>-1.1</v>
       </c>
       <c r="L24" t="n">
-        <v>80.59999999999999</v>
+        <v>146.492</v>
       </c>
       <c r="M24" t="n">
-        <v>9.6</v>
+        <v>5.514</v>
       </c>
       <c r="P24" t="n">
-        <v>57</v>
+        <v>41.5</v>
       </c>
       <c r="Q24" t="n">
-        <v>-4.2</v>
+        <v>-2.9</v>
+      </c>
+      <c r="X24" t="n">
+        <v>-3.03</v>
       </c>
       <c r="Y24" t="n">
-        <v>-10.9</v>
+        <v>-2.8</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>75.541</v>
       </c>
       <c r="AA24" t="n">
-        <v>4.92</v>
+        <v>-14.36</v>
       </c>
       <c r="AB24" t="n">
-        <v>16.7</v>
-      </c>
-      <c r="AC24" t="n">
-        <v>0.50625</v>
+        <v>0.4</v>
       </c>
       <c r="AF24" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>reports/iraq-sovereign-credit.md</t>
+          <t>reports/indonesia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Middle East</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>B-</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Caa1</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>None active (Article IV surveillance and Post-Financing Assessment; last SBA expired 2018)</t>
+        </is>
+      </c>
       <c r="G25" t="n">
-        <v>3.5</v>
+        <v>-6.8</v>
       </c>
       <c r="H25" t="n">
-        <v>1.54</v>
-      </c>
-      <c r="I25" t="n">
-        <v>3.25</v>
-      </c>
-      <c r="J25" t="n">
-        <v>1.71</v>
+        <v>3.0928</v>
       </c>
       <c r="K25" t="n">
-        <v>1.9</v>
+        <v>-5.3</v>
       </c>
       <c r="L25" t="n">
-        <v>241.63</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="M25" t="n">
-        <v>14.36</v>
+        <v>9.6</v>
       </c>
       <c r="P25" t="n">
-        <v>69.8</v>
+        <v>57</v>
       </c>
       <c r="Q25" t="n">
-        <v>-5.9</v>
-      </c>
-      <c r="X25" t="n">
-        <v>2.67</v>
+        <v>-4.2</v>
       </c>
       <c r="Y25" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="Z25" t="n">
-        <v>232.204</v>
+        <v>-10.9</v>
       </c>
       <c r="AA25" t="n">
-        <v>4.53</v>
+        <v>4.92</v>
       </c>
       <c r="AB25" t="n">
-        <v>-1.6</v>
+        <v>16.7</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>0.50625</v>
       </c>
       <c r="AF25" t="inlineStr">
         <is>
@@ -2203,85 +2161,63 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>reports/israel-sovereign-credit.md</t>
+          <t>reports/iraq-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Middle East (CEEMEA)</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Ba3</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Extended Fund Facility (4-year, SDR 926.37m; Fifth Review completed Jun-26, with RSF)</t>
-        </is>
-      </c>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
       <c r="G26" t="n">
-        <v>2.7</v>
+        <v>3.5</v>
       </c>
       <c r="H26" t="n">
-        <v>2.7011</v>
+        <v>1.54</v>
       </c>
       <c r="I26" t="n">
-        <v>6</v>
+        <v>3.25</v>
       </c>
       <c r="J26" t="n">
-        <v>3.3</v>
+        <v>1.71</v>
       </c>
       <c r="K26" t="n">
-        <v>-6.2</v>
+        <v>1.9</v>
       </c>
       <c r="L26" t="n">
-        <v>28.5</v>
+        <v>241.63</v>
       </c>
       <c r="M26" t="n">
-        <v>9.199999999999999</v>
+        <v>14.36</v>
       </c>
       <c r="P26" t="n">
-        <v>83.59999999999999</v>
+        <v>69.8</v>
       </c>
       <c r="Q26" t="n">
-        <v>-5.2</v>
-      </c>
-      <c r="R26" t="n">
-        <v>-2.8</v>
+        <v>-5.9</v>
+      </c>
+      <c r="X26" t="n">
+        <v>2.67</v>
       </c>
       <c r="Y26" t="n">
-        <v>23</v>
+        <v>4.9</v>
       </c>
       <c r="Z26" t="n">
-        <v>21.01</v>
+        <v>232.204</v>
       </c>
       <c r="AA26" t="n">
-        <v>-3.11</v>
+        <v>4.53</v>
       </c>
       <c r="AB26" t="n">
-        <v>-6.1</v>
-      </c>
-      <c r="AC26" t="n">
-        <v>3.95</v>
+        <v>-1.6</v>
       </c>
       <c r="AF26" t="inlineStr">
         <is>
@@ -2290,75 +2226,85 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>reports/jordan-sovereign-credit.md</t>
+          <t>reports/israel-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CIS / Central Asia</t>
+          <t>Middle East (CEEMEA)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>BBB</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Baa1</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
+          <t>Ba3</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Extended Fund Facility (4-year, SDR 926.37m; Fifth Review completed Jun-26, with RSF)</t>
+        </is>
+      </c>
       <c r="G27" t="n">
-        <v>4.6</v>
+        <v>2.7</v>
       </c>
       <c r="H27" t="n">
-        <v>9.24</v>
+        <v>2.7011</v>
       </c>
       <c r="I27" t="n">
-        <v>16.75</v>
+        <v>6</v>
       </c>
       <c r="J27" t="n">
-        <v>7.51</v>
+        <v>3.3</v>
       </c>
       <c r="K27" t="n">
-        <v>-1</v>
+        <v>-6.2</v>
       </c>
       <c r="L27" t="n">
-        <v>70.56999999999999</v>
+        <v>28.5</v>
       </c>
       <c r="M27" t="n">
-        <v>7.39</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="P27" t="n">
-        <v>24.9</v>
+        <v>83.59999999999999</v>
       </c>
       <c r="Q27" t="n">
-        <v>-1.3</v>
+        <v>-5.2</v>
+      </c>
+      <c r="R27" t="n">
+        <v>-2.8</v>
       </c>
       <c r="Y27" t="n">
-        <v>29.9</v>
+        <v>23</v>
       </c>
       <c r="Z27" t="n">
-        <v>59.792</v>
+        <v>21.01</v>
       </c>
       <c r="AA27" t="n">
-        <v>-13.41</v>
+        <v>-3.11</v>
       </c>
       <c r="AB27" t="n">
-        <v>11.5</v>
+        <v>-6.1</v>
+      </c>
+      <c r="AC27" t="n">
+        <v>3.95</v>
       </c>
       <c r="AF27" t="inlineStr">
         <is>
@@ -2367,76 +2313,75 @@
       </c>
       <c r="AG27" t="inlineStr">
         <is>
-          <t>reports/kazakhstan-sovereign-credit.md</t>
+          <t>reports/jordan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>CIS / Central Asia</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>B-</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>BBB</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>B3</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25, successor talks ongoing</t>
-        </is>
-      </c>
+          <t>Baa1</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
       <c r="G28" t="n">
-        <v>4.5</v>
+        <v>4.6</v>
       </c>
       <c r="H28" t="n">
-        <v>6.76</v>
+        <v>9.24</v>
       </c>
       <c r="I28" t="n">
-        <v>8.75</v>
+        <v>16.75</v>
       </c>
       <c r="J28" t="n">
-        <v>1.99</v>
+        <v>7.51</v>
       </c>
       <c r="K28" t="n">
-        <v>-4.1</v>
+        <v>-1</v>
       </c>
       <c r="L28" t="n">
-        <v>14.702</v>
+        <v>70.56999999999999</v>
       </c>
       <c r="M28" t="n">
-        <v>4.632</v>
+        <v>7.39</v>
       </c>
       <c r="P28" t="n">
-        <v>68.5</v>
+        <v>24.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>-6.4</v>
-      </c>
-      <c r="S28" t="n">
-        <v>33</v>
+        <v>-1.3</v>
       </c>
       <c r="Y28" t="n">
-        <v>34.7</v>
+        <v>29.9</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>59.792</v>
+      </c>
+      <c r="AA28" t="n">
+        <v>-13.41</v>
       </c>
       <c r="AB28" t="n">
-        <v>-2.9</v>
+        <v>11.5</v>
       </c>
       <c r="AF28" t="inlineStr">
         <is>
@@ -2445,72 +2390,76 @@
       </c>
       <c r="AG28" t="inlineStr">
         <is>
-          <t>reports/kenya-sovereign-credit.md</t>
+          <t>reports/kazakhstan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Middle East (GCC)</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>A1</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>None; prior EFF/ECF/RSF expired uncompleted Apr-25, successor talks ongoing</t>
+        </is>
+      </c>
       <c r="G29" t="n">
-        <v>-0.6</v>
+        <v>4.5</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>6.76</v>
       </c>
       <c r="I29" t="n">
-        <v>3.5</v>
+        <v>8.75</v>
       </c>
       <c r="J29" t="n">
-        <v>3.5</v>
+        <v>1.99</v>
       </c>
       <c r="K29" t="n">
-        <v>18.8</v>
+        <v>-4.1</v>
       </c>
       <c r="L29" t="n">
-        <v>32.689</v>
+        <v>14.702</v>
       </c>
       <c r="M29" t="n">
-        <v>8.4</v>
+        <v>4.632</v>
       </c>
       <c r="P29" t="n">
-        <v>2.9</v>
+        <v>68.5</v>
       </c>
       <c r="Q29" t="n">
-        <v>-18.5</v>
+        <v>-6.4</v>
+      </c>
+      <c r="S29" t="n">
+        <v>33</v>
       </c>
       <c r="Y29" t="n">
-        <v>-23.4</v>
-      </c>
-      <c r="AA29" t="n">
-        <v>32.54</v>
+        <v>34.7</v>
       </c>
       <c r="AB29" t="n">
-        <v>28.1</v>
+        <v>-2.9</v>
       </c>
       <c r="AF29" t="inlineStr">
         <is>
@@ -2519,55 +2468,72 @@
       </c>
       <c r="AG29" t="inlineStr">
         <is>
-          <t>reports/kuwait-sovereign-credit.md</t>
+          <t>reports/kenya-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MENA</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>None; mission of 15-18 Sep-26 ended without staff-level agreement</t>
-        </is>
-      </c>
+          <t>Middle East (GCC)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>AA-</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="n">
-        <v>4</v>
+        <v>-0.6</v>
       </c>
       <c r="H30" t="n">
-        <v>16.66</v>
+        <v>0</v>
+      </c>
+      <c r="I30" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="J30" t="n">
+        <v>3.5</v>
       </c>
       <c r="K30" t="n">
-        <v>-22.5</v>
+        <v>18.8</v>
       </c>
       <c r="L30" t="n">
-        <v>38.16</v>
+        <v>32.689</v>
       </c>
       <c r="M30" t="n">
-        <v>13.6</v>
+        <v>8.4</v>
       </c>
       <c r="P30" t="n">
-        <v>139.4</v>
+        <v>2.9</v>
       </c>
       <c r="Q30" t="n">
-        <v>3.3</v>
+        <v>-18.5</v>
       </c>
       <c r="Y30" t="n">
-        <v>31.2</v>
+        <v>-23.4</v>
       </c>
       <c r="AA30" t="n">
-        <v>-9.16</v>
+        <v>32.54</v>
       </c>
       <c r="AB30" t="n">
-        <v>-4.6</v>
+        <v>28.1</v>
       </c>
       <c r="AF30" t="inlineStr">
         <is>
@@ -2576,128 +2542,120 @@
       </c>
       <c r="AG30" t="inlineStr">
         <is>
-          <t>reports/lebanon-sovereign-credit.md</t>
+          <t>reports/kuwait-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Asia</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr"/>
+          <t>MENA</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>None; mission of 15-18 Sep-26 ended without staff-level agreement</t>
+        </is>
+      </c>
       <c r="G31" t="n">
-        <v>4.7</v>
+        <v>4</v>
       </c>
       <c r="H31" t="n">
-        <v>1.7817</v>
-      </c>
-      <c r="I31" t="n">
-        <v>2.75</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.97</v>
+        <v>16.66</v>
       </c>
       <c r="K31" t="n">
-        <v>1.4</v>
+        <v>-22.5</v>
       </c>
       <c r="L31" t="n">
-        <v>131.981</v>
+        <v>38.16</v>
       </c>
       <c r="M31" t="n">
-        <v>4.276</v>
+        <v>13.6</v>
       </c>
       <c r="P31" t="n">
-        <v>69.5</v>
+        <v>139.4</v>
       </c>
       <c r="Q31" t="n">
-        <v>-3.3</v>
-      </c>
-      <c r="X31" t="n">
-        <v>1.2</v>
+        <v>3.3</v>
       </c>
       <c r="Y31" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="Z31" t="n">
-        <v>97.798</v>
+        <v>31.2</v>
       </c>
       <c r="AA31" t="n">
-        <v>10.37</v>
+        <v>-9.16</v>
       </c>
       <c r="AB31" t="n">
-        <v>1</v>
+        <v>-4.6</v>
       </c>
       <c r="AF31" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG31" t="inlineStr">
         <is>
-          <t>reports/malaysia-sovereign-credit.md</t>
+          <t>reports/lebanon-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Latin America</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
       <c r="G32" t="n">
-        <v>1.6</v>
+        <v>4.7</v>
       </c>
       <c r="H32" t="n">
-        <v>3.2619</v>
+        <v>1.7817</v>
       </c>
       <c r="I32" t="n">
-        <v>6.5</v>
+        <v>2.75</v>
       </c>
       <c r="J32" t="n">
-        <v>3.24</v>
+        <v>0.97</v>
       </c>
       <c r="K32" t="n">
-        <v>-0.4</v>
+        <v>1.4</v>
       </c>
       <c r="L32" t="n">
-        <v>265.969</v>
+        <v>131.981</v>
       </c>
       <c r="M32" t="n">
-        <v>3.73</v>
+        <v>4.276</v>
       </c>
       <c r="P32" t="n">
-        <v>62.7</v>
+        <v>69.5</v>
       </c>
       <c r="Q32" t="n">
-        <v>-4.4</v>
+        <v>-3.3</v>
       </c>
       <c r="X32" t="n">
-        <v>1.8</v>
+        <v>1.2</v>
       </c>
       <c r="Y32" t="n">
-        <v>6.8</v>
+        <v>7.5</v>
       </c>
       <c r="Z32" t="n">
-        <v>250.968</v>
+        <v>97.798</v>
       </c>
       <c r="AA32" t="n">
-        <v>-0.7</v>
+        <v>10.37</v>
       </c>
       <c r="AB32" t="n">
-        <v>0.3</v>
+        <v>1</v>
       </c>
       <c r="AF32" t="inlineStr">
         <is>
@@ -2706,138 +2664,116 @@
       </c>
       <c r="AG32" t="inlineStr">
         <is>
-          <t>reports/mexico-sovereign-credit.md</t>
+          <t>reports/malaysia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Montenegro</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Western Balkans (CEEMEA)</t>
+          <t>Latin America</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
       <c r="G33" t="n">
-        <v>2.8</v>
+        <v>1.6</v>
       </c>
       <c r="H33" t="n">
-        <v>3.6043</v>
+        <v>3.2619</v>
+      </c>
+      <c r="I33" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J33" t="n">
+        <v>3.24</v>
       </c>
       <c r="K33" t="n">
-        <v>-19.4</v>
+        <v>-0.4</v>
       </c>
       <c r="L33" t="n">
-        <v>2.196</v>
+        <v>265.969</v>
       </c>
       <c r="M33" t="n">
-        <v>3.947</v>
+        <v>3.73</v>
       </c>
       <c r="P33" t="n">
-        <v>63.5</v>
+        <v>62.7</v>
       </c>
       <c r="Q33" t="n">
-        <v>-4</v>
+        <v>-4.4</v>
+      </c>
+      <c r="X33" t="n">
+        <v>1.8</v>
       </c>
       <c r="Y33" t="n">
-        <v>26.1</v>
+        <v>6.8</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>250.968</v>
       </c>
       <c r="AA33" t="n">
-        <v>-2.07</v>
+        <v>-0.7</v>
       </c>
       <c r="AB33" t="n">
-        <v>-1.6</v>
+        <v>0.3</v>
       </c>
       <c r="AF33" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG33" t="inlineStr">
         <is>
-          <t>reports/montenegro-sovereign-credit.md</t>
+          <t>reports/mexico-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>North Africa</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>BB+</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Ba1</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Flexible Credit Line (2-year, precautionary); Mid-Term Review completed Mar-26; RSF SDR 1.0bn approved Sep-23</t>
-        </is>
-      </c>
+          <t>Western Balkans (CEEMEA)</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="n">
-        <v>4.9</v>
+        <v>2.8</v>
       </c>
       <c r="H34" t="n">
-        <v>-0.3333</v>
-      </c>
-      <c r="I34" t="n">
-        <v>2.25</v>
-      </c>
-      <c r="J34" t="n">
-        <v>2.58</v>
+        <v>3.6043</v>
       </c>
       <c r="K34" t="n">
-        <v>-3.1</v>
+        <v>-19.4</v>
       </c>
       <c r="L34" t="n">
-        <v>55.65</v>
+        <v>2.196</v>
       </c>
       <c r="M34" t="n">
-        <v>5.5</v>
+        <v>3.947</v>
       </c>
       <c r="P34" t="n">
-        <v>67.2</v>
+        <v>63.5</v>
       </c>
       <c r="Q34" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="S34" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="X34" t="n">
-        <v>-2.1</v>
+        <v>-4</v>
       </c>
       <c r="Y34" t="n">
-        <v>18</v>
-      </c>
-      <c r="Z34" t="n">
-        <v>50.756</v>
+        <v>26.1</v>
       </c>
       <c r="AA34" t="n">
-        <v>-5.83</v>
+        <v>-2.07</v>
       </c>
       <c r="AB34" t="n">
-        <v>-3.2</v>
+        <v>-1.6</v>
       </c>
       <c r="AF34" t="inlineStr">
         <is>
@@ -2846,79 +2782,85 @@
       </c>
       <c r="AG34" t="inlineStr">
         <is>
-          <t>reports/morocco-sovereign-credit.md</t>
+          <t>reports/montenegro-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Mozambique</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Africa</t>
+          <t>North Africa</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CC</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>CCC (LC: SD)</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Caa3</t>
+          <t>Ba1</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>None; 2022 ECF (SDR 340.8m) lapsed Apr-25; successor arrangement under discussion after Sep-26 staff mission</t>
+          <t>Flexible Credit Line (2-year, precautionary); Mid-Term Review completed Mar-26; RSF SDR 1.0bn approved Sep-23</t>
         </is>
       </c>
       <c r="G35" t="n">
-        <v>0.5</v>
+        <v>4.9</v>
       </c>
       <c r="H35" t="n">
-        <v>6.5</v>
+        <v>-0.3333</v>
       </c>
       <c r="I35" t="n">
-        <v>9.25</v>
+        <v>2.25</v>
       </c>
       <c r="J35" t="n">
-        <v>2.75</v>
+        <v>2.58</v>
       </c>
       <c r="K35" t="n">
-        <v>-43</v>
+        <v>-3.1</v>
       </c>
       <c r="L35" t="n">
-        <v>3.9</v>
+        <v>55.65</v>
       </c>
       <c r="M35" t="n">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="P35" t="n">
-        <v>94</v>
+        <v>67.2</v>
       </c>
       <c r="Q35" t="n">
-        <v>-6.5</v>
+        <v>-3.5</v>
+      </c>
+      <c r="S35" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="X35" t="n">
+        <v>-2.1</v>
       </c>
       <c r="Y35" t="n">
-        <v>4.9</v>
+        <v>18</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>50.756</v>
       </c>
       <c r="AA35" t="n">
-        <v>-2.95</v>
+        <v>-5.83</v>
       </c>
       <c r="AB35" t="n">
-        <v>-0.1</v>
-      </c>
-      <c r="AC35" t="n">
-        <v>0.9</v>
+        <v>-3.2</v>
       </c>
       <c r="AF35" t="inlineStr">
         <is>
@@ -2927,14 +2869,14 @@
       </c>
       <c r="AG35" t="inlineStr">
         <is>
-          <t>reports/mozambique-sovereign-credit.md</t>
+          <t>reports/morocco-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Namibia</t>
+          <t>Mozambique</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2942,39 +2884,64 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="F36" t="inlineStr"/>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>CC</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>CCC (LC: SD)</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Caa3</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>None; 2022 ECF (SDR 340.8m) lapsed Apr-25; successor arrangement under discussion after Sep-26 staff mission</t>
+        </is>
+      </c>
       <c r="G36" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="H36" t="n">
-        <v>4.4106</v>
+        <v>6.5</v>
+      </c>
+      <c r="I36" t="n">
+        <v>9.25</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2.75</v>
       </c>
       <c r="K36" t="n">
-        <v>-15.7</v>
+        <v>-43</v>
       </c>
       <c r="L36" t="n">
-        <v>3.252</v>
+        <v>3.9</v>
       </c>
       <c r="M36" t="n">
-        <v>3.958</v>
+        <v>6.5</v>
       </c>
       <c r="P36" t="n">
-        <v>70.5</v>
+        <v>94</v>
       </c>
       <c r="Q36" t="n">
-        <v>-6.1</v>
+        <v>-6.5</v>
       </c>
       <c r="Y36" t="n">
-        <v>-6.3</v>
-      </c>
-      <c r="Z36" t="n">
-        <v>2.151</v>
+        <v>4.9</v>
       </c>
       <c r="AA36" t="n">
-        <v>-1.86</v>
+        <v>-2.95</v>
       </c>
       <c r="AB36" t="n">
-        <v>0.8</v>
+        <v>-0.1</v>
+      </c>
+      <c r="AC36" t="n">
+        <v>0.9</v>
       </c>
       <c r="AF36" t="inlineStr">
         <is>
@@ -2983,84 +2950,54 @@
       </c>
       <c r="AG36" t="inlineStr">
         <is>
-          <t>reports/namibia-sovereign-credit.md</t>
+          <t>reports/mozambique-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Namibia</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
-        </is>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>B3</t>
+          <t>Africa</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
       <c r="G37" t="n">
-        <v>4.1</v>
+        <v>2.4</v>
       </c>
       <c r="H37" t="n">
-        <v>15.39</v>
-      </c>
-      <c r="I37" t="n">
-        <v>23</v>
-      </c>
-      <c r="J37" t="n">
-        <v>7.61</v>
+        <v>4.4106</v>
       </c>
       <c r="K37" t="n">
-        <v>5.8</v>
+        <v>-15.7</v>
       </c>
       <c r="L37" t="n">
-        <v>54.98</v>
+        <v>3.252</v>
       </c>
       <c r="M37" t="n">
-        <v>9.199999999999999</v>
-      </c>
-      <c r="O37" t="n">
-        <v>14.4</v>
+        <v>3.958</v>
       </c>
       <c r="P37" t="n">
-        <v>32.3</v>
+        <v>70.5</v>
       </c>
       <c r="Q37" t="n">
-        <v>-4.4</v>
-      </c>
-      <c r="S37" t="n">
-        <v>55</v>
-      </c>
-      <c r="X37" t="n">
-        <v>-0.51</v>
+        <v>-6.1</v>
       </c>
       <c r="Y37" t="n">
-        <v>30.8</v>
+        <v>-6.3</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>2.151</v>
       </c>
       <c r="AA37" t="n">
-        <v>15.61</v>
+        <v>-1.86</v>
       </c>
       <c r="AB37" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="AC37" t="n">
-        <v>15.12</v>
+        <v>0.8</v>
       </c>
       <c r="AF37" t="inlineStr">
         <is>
@@ -3069,80 +3006,84 @@
       </c>
       <c r="AG37" t="inlineStr">
         <is>
-          <t>reports/nigeria-sovereign-credit.md</t>
+          <t>reports/namibia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CEEMEA - Western Balkans</t>
+          <t>Sub-Saharan Africa</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BB+</t>
+          <t>B</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="F38" t="inlineStr">
-        <is>
-          <t>PLL concluded Nov-24</t>
-        </is>
-      </c>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr"/>
       <c r="G38" t="n">
-        <v>3.1</v>
+        <v>4.1</v>
       </c>
       <c r="H38" t="n">
-        <v>2.5729</v>
+        <v>15.39</v>
       </c>
       <c r="I38" t="n">
-        <v>4.25</v>
+        <v>23</v>
       </c>
       <c r="J38" t="n">
-        <v>1.68</v>
+        <v>7.61</v>
       </c>
       <c r="K38" t="n">
-        <v>-5</v>
+        <v>5.8</v>
       </c>
       <c r="L38" t="n">
-        <v>5.51</v>
+        <v>54.98</v>
       </c>
       <c r="M38" t="n">
-        <v>4.2</v>
+        <v>9.199999999999999</v>
+      </c>
+      <c r="O38" t="n">
+        <v>14.4</v>
       </c>
       <c r="P38" t="n">
-        <v>55.2</v>
+        <v>32.3</v>
       </c>
       <c r="Q38" t="n">
-        <v>-4.2</v>
+        <v>-4.4</v>
+      </c>
+      <c r="S38" t="n">
+        <v>55</v>
       </c>
       <c r="X38" t="n">
-        <v>1.52</v>
+        <v>-0.51</v>
       </c>
       <c r="Y38" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="Z38" t="n">
-        <v>4.474</v>
+        <v>30.8</v>
       </c>
       <c r="AA38" t="n">
-        <v>-0.99</v>
+        <v>15.61</v>
       </c>
       <c r="AB38" t="n">
-        <v>-2.6</v>
+        <v>4.6</v>
       </c>
       <c r="AC38" t="n">
-        <v>2.16</v>
+        <v>15.12</v>
       </c>
       <c r="AF38" t="inlineStr">
         <is>
@@ -3151,67 +3092,80 @@
       </c>
       <c r="AG38" t="inlineStr">
         <is>
-          <t>reports/north-macedonia-sovereign-credit.md</t>
+          <t>reports/nigeria-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Oman</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Middle East (GCC)</t>
+          <t>CEEMEA - Western Balkans</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>BBB-</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Baa3</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>PLL concluded Nov-24</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>2.1</v>
+        <v>3.1</v>
       </c>
       <c r="H39" t="n">
-        <v>3.3771</v>
+        <v>2.5729</v>
+      </c>
+      <c r="I39" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1.68</v>
       </c>
       <c r="K39" t="n">
-        <v>2.5</v>
+        <v>-5</v>
       </c>
       <c r="L39" t="n">
-        <v>18.38</v>
+        <v>5.51</v>
       </c>
       <c r="M39" t="n">
-        <v>5</v>
+        <v>4.2</v>
       </c>
       <c r="P39" t="n">
-        <v>34.7</v>
+        <v>55.2</v>
       </c>
       <c r="Q39" t="n">
-        <v>0.6</v>
+        <v>-4.2</v>
+      </c>
+      <c r="X39" t="n">
+        <v>1.52</v>
       </c>
       <c r="Y39" t="n">
-        <v>9.199999999999999</v>
+        <v>7.2</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>4.474</v>
+      </c>
+      <c r="AA39" t="n">
+        <v>-0.99</v>
       </c>
       <c r="AB39" t="n">
-        <v>15.6</v>
+        <v>-2.6</v>
+      </c>
+      <c r="AC39" t="n">
+        <v>2.16</v>
       </c>
       <c r="AF39" t="inlineStr">
         <is>
@@ -3220,54 +3174,67 @@
       </c>
       <c r="AG39" t="inlineStr">
         <is>
-          <t>reports/oman-sovereign-credit.md</t>
+          <t>reports/north-macedonia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Oman</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>South Asia</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr"/>
+          <t>Middle East (GCC)</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>BBB-</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Baa3</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
       <c r="G40" t="n">
-        <v>3.6</v>
+        <v>2.1</v>
       </c>
       <c r="H40" t="n">
-        <v>10.2591</v>
+        <v>3.3771</v>
       </c>
       <c r="K40" t="n">
-        <v>-0.4</v>
+        <v>2.5</v>
       </c>
       <c r="L40" t="n">
-        <v>27.993</v>
+        <v>18.38</v>
       </c>
       <c r="M40" t="n">
-        <v>3.755</v>
+        <v>5</v>
       </c>
       <c r="P40" t="n">
-        <v>70.09999999999999</v>
+        <v>34.7</v>
       </c>
       <c r="Q40" t="n">
-        <v>-3.2</v>
-      </c>
-      <c r="X40" t="n">
-        <v>1.02</v>
+        <v>0.6</v>
       </c>
       <c r="Y40" t="n">
-        <v>22.8</v>
-      </c>
-      <c r="AA40" t="n">
-        <v>-0.14</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="AB40" t="n">
-        <v>-2.3</v>
+        <v>15.6</v>
       </c>
       <c r="AF40" t="inlineStr">
         <is>
@@ -3276,128 +3243,119 @@
       </c>
       <c r="AG40" t="inlineStr">
         <is>
-          <t>reports/pakistan-sovereign-credit.md</t>
+          <t>reports/oman-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Latin America</t>
+          <t>South Asia</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
       <c r="G41" t="n">
-        <v>2.8</v>
+        <v>3.6</v>
       </c>
       <c r="H41" t="n">
-        <v>4.0636</v>
-      </c>
-      <c r="I41" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="J41" t="n">
-        <v>0.19</v>
+        <v>10.2591</v>
       </c>
       <c r="K41" t="n">
-        <v>3.4</v>
+        <v>-0.4</v>
       </c>
       <c r="L41" t="n">
-        <v>95.26900000000001</v>
+        <v>27.993</v>
       </c>
       <c r="M41" t="n">
-        <v>10.423</v>
+        <v>3.755</v>
       </c>
       <c r="P41" t="n">
-        <v>30</v>
+        <v>70.09999999999999</v>
       </c>
       <c r="Q41" t="n">
-        <v>-2</v>
+        <v>-3.2</v>
       </c>
       <c r="X41" t="n">
-        <v>1.8</v>
+        <v>1.02</v>
       </c>
       <c r="Y41" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="Z41" t="n">
-        <v>87.288</v>
+        <v>22.8</v>
       </c>
       <c r="AA41" t="n">
-        <v>12.01</v>
+        <v>-0.14</v>
       </c>
       <c r="AB41" t="n">
-        <v>2.5</v>
+        <v>-2.3</v>
       </c>
       <c r="AF41" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG41" t="inlineStr">
         <is>
-          <t>reports/peru-sovereign-credit.md</t>
+          <t>reports/pakistan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Philippines</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Latin America</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
       <c r="G42" t="n">
-        <v>4.1</v>
+        <v>2.8</v>
       </c>
       <c r="H42" t="n">
-        <v>6.3629</v>
+        <v>4.0636</v>
       </c>
       <c r="I42" t="n">
-        <v>5</v>
+        <v>4.25</v>
       </c>
       <c r="J42" t="n">
-        <v>-1.36</v>
+        <v>0.19</v>
       </c>
       <c r="K42" t="n">
-        <v>-4.4</v>
+        <v>3.4</v>
       </c>
       <c r="L42" t="n">
-        <v>103.316</v>
+        <v>95.26900000000001</v>
       </c>
       <c r="M42" t="n">
-        <v>7.306</v>
+        <v>10.423</v>
       </c>
       <c r="P42" t="n">
-        <v>60.2</v>
+        <v>30</v>
       </c>
       <c r="Q42" t="n">
-        <v>-3.7</v>
+        <v>-2</v>
       </c>
       <c r="X42" t="n">
-        <v>-0.19</v>
+        <v>1.8</v>
       </c>
       <c r="Y42" t="n">
-        <v>-2</v>
+        <v>16.3</v>
       </c>
       <c r="Z42" t="n">
-        <v>93.018</v>
+        <v>87.288</v>
       </c>
       <c r="AA42" t="n">
-        <v>-22.11</v>
+        <v>12.01</v>
       </c>
       <c r="AB42" t="n">
-        <v>-1.4</v>
+        <v>2.5</v>
       </c>
       <c r="AF42" t="inlineStr">
         <is>
@@ -3406,63 +3364,63 @@
       </c>
       <c r="AG42" t="inlineStr">
         <is>
-          <t>reports/philippines-sovereign-credit.md</t>
+          <t>reports/peru-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Philippines</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Central Europe</t>
+          <t>Asia</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
       <c r="G43" t="n">
-        <v>3.3</v>
+        <v>4.1</v>
       </c>
       <c r="H43" t="n">
-        <v>3.2123</v>
+        <v>6.3629</v>
       </c>
       <c r="I43" t="n">
-        <v>3.75</v>
+        <v>5</v>
       </c>
       <c r="J43" t="n">
-        <v>0.54</v>
+        <v>-1.36</v>
       </c>
       <c r="K43" t="n">
-        <v>-1.1</v>
+        <v>-4.4</v>
       </c>
       <c r="L43" t="n">
-        <v>304.971</v>
+        <v>103.316</v>
       </c>
       <c r="M43" t="n">
-        <v>5.861</v>
+        <v>7.306</v>
       </c>
       <c r="P43" t="n">
-        <v>65.7</v>
+        <v>60.2</v>
       </c>
       <c r="Q43" t="n">
-        <v>-6.7</v>
+        <v>-3.7</v>
       </c>
       <c r="X43" t="n">
-        <v>1.5</v>
+        <v>-0.19</v>
       </c>
       <c r="Y43" t="n">
-        <v>16.9</v>
+        <v>-2</v>
       </c>
       <c r="Z43" t="n">
-        <v>277.21</v>
+        <v>93.018</v>
       </c>
       <c r="AA43" t="n">
-        <v>-13.87</v>
+        <v>-22.11</v>
       </c>
       <c r="AB43" t="n">
-        <v>-1.1</v>
+        <v>-1.4</v>
       </c>
       <c r="AF43" t="inlineStr">
         <is>
@@ -3471,279 +3429,279 @@
       </c>
       <c r="AG43" t="inlineStr">
         <is>
-          <t>reports/poland-sovereign-credit.md</t>
+          <t>reports/philippines-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>GCC</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>AA</t>
+          <t>Central Europe</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
       <c r="G44" t="n">
-        <v>-8.6</v>
+        <v>3.3</v>
       </c>
       <c r="H44" t="n">
-        <v>0.73</v>
+        <v>3.2123</v>
       </c>
       <c r="I44" t="n">
-        <v>4.35</v>
+        <v>3.75</v>
       </c>
       <c r="J44" t="n">
-        <v>3.62</v>
+        <v>0.54</v>
       </c>
       <c r="K44" t="n">
-        <v>11</v>
+        <v>-1.1</v>
       </c>
       <c r="L44" t="n">
-        <v>61.1</v>
+        <v>304.971</v>
       </c>
       <c r="M44" t="n">
-        <v>7.45</v>
+        <v>5.861</v>
       </c>
       <c r="P44" t="n">
-        <v>43.3</v>
+        <v>65.7</v>
       </c>
       <c r="Q44" t="n">
-        <v>-3.4</v>
+        <v>-6.7</v>
+      </c>
+      <c r="X44" t="n">
+        <v>1.5</v>
       </c>
       <c r="Y44" t="n">
-        <v>10.4</v>
+        <v>16.9</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>277.21</v>
       </c>
       <c r="AA44" t="n">
-        <v>28.52</v>
+        <v>-13.87</v>
       </c>
       <c r="AB44" t="n">
-        <v>14.7</v>
+        <v>-1.1</v>
       </c>
       <c r="AF44" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG44" t="inlineStr">
         <is>
-          <t>reports/qatar-sovereign-credit.md</t>
+          <t>reports/poland-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Central Europe</t>
+          <t>GCC</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>AA</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
       <c r="G45" t="n">
-        <v>0.7</v>
+        <v>-8.6</v>
       </c>
       <c r="H45" t="n">
-        <v>8.16</v>
+        <v>0.73</v>
       </c>
       <c r="I45" t="n">
-        <v>6.5</v>
+        <v>4.35</v>
       </c>
       <c r="J45" t="n">
-        <v>-1.66</v>
+        <v>3.62</v>
       </c>
       <c r="K45" t="n">
-        <v>-6.8</v>
+        <v>11</v>
       </c>
       <c r="L45" t="n">
-        <v>90.04300000000001</v>
+        <v>61.1</v>
       </c>
       <c r="M45" t="n">
-        <v>5.528</v>
+        <v>7.45</v>
       </c>
       <c r="P45" t="n">
-        <v>61.9</v>
+        <v>43.3</v>
       </c>
       <c r="Q45" t="n">
-        <v>-6.2</v>
-      </c>
-      <c r="X45" t="n">
-        <v>1.95</v>
+        <v>-3.4</v>
       </c>
       <c r="Y45" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="Z45" t="n">
-        <v>72.172</v>
+        <v>10.4</v>
       </c>
       <c r="AA45" t="n">
-        <v>-32.2</v>
+        <v>28.52</v>
       </c>
       <c r="AB45" t="n">
-        <v>-0.5</v>
+        <v>14.7</v>
       </c>
       <c r="AF45" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG45" t="inlineStr">
         <is>
-          <t>reports/romania-sovereign-credit.md</t>
+          <t>reports/qatar-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Rwanda</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr">
-        <is>
-          <t>B+</t>
-        </is>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>38-month ECF (reported)</t>
-        </is>
-      </c>
+          <t>Central Europe</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr"/>
       <c r="G46" t="n">
-        <v>9.699999999999999</v>
+        <v>0.7</v>
       </c>
       <c r="H46" t="n">
-        <v>15.7</v>
+        <v>8.16</v>
       </c>
       <c r="I46" t="n">
-        <v>8.75</v>
+        <v>6.5</v>
       </c>
       <c r="J46" t="n">
-        <v>-6.95</v>
+        <v>-1.66</v>
       </c>
       <c r="K46" t="n">
-        <v>-15</v>
+        <v>-6.8</v>
       </c>
       <c r="L46" t="n">
-        <v>2.2</v>
+        <v>90.04300000000001</v>
       </c>
       <c r="M46" t="n">
-        <v>4</v>
-      </c>
-      <c r="O46" t="n">
-        <v>63</v>
+        <v>5.528</v>
       </c>
       <c r="P46" t="n">
-        <v>77.5</v>
+        <v>61.9</v>
       </c>
       <c r="Q46" t="n">
-        <v>-4.8</v>
+        <v>-6.2</v>
+      </c>
+      <c r="X46" t="n">
+        <v>1.95</v>
       </c>
       <c r="Y46" t="n">
-        <v>-16.4</v>
+        <v>2.9</v>
       </c>
       <c r="Z46" t="n">
-        <v>1.795</v>
+        <v>72.172</v>
       </c>
       <c r="AA46" t="n">
-        <v>-1.98</v>
+        <v>-32.2</v>
       </c>
       <c r="AB46" t="n">
-        <v>-0</v>
-      </c>
-      <c r="AC46" t="n">
-        <v>0.62</v>
+        <v>-0.5</v>
       </c>
       <c r="AF46" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG46" t="inlineStr">
         <is>
-          <t>reports/rwanda-sovereign-credit.md</t>
+          <t>reports/romania-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Rwanda</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Middle East</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr"/>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>B+</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>38-month ECF (reported)</t>
+        </is>
+      </c>
       <c r="G47" t="n">
-        <v>3.1</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="H47" t="n">
-        <v>1.82</v>
+        <v>15.7</v>
       </c>
       <c r="I47" t="n">
-        <v>4.5</v>
+        <v>8.75</v>
       </c>
       <c r="J47" t="n">
-        <v>2.68</v>
+        <v>-6.95</v>
       </c>
       <c r="K47" t="n">
-        <v>-1.6</v>
+        <v>-15</v>
       </c>
       <c r="L47" t="n">
-        <v>488.684</v>
+        <v>2.2</v>
       </c>
       <c r="M47" t="n">
-        <v>15.6</v>
+        <v>4</v>
+      </c>
+      <c r="O47" t="n">
+        <v>63</v>
       </c>
       <c r="P47" t="n">
-        <v>32.1</v>
+        <v>77.5</v>
       </c>
       <c r="Q47" t="n">
-        <v>-3.5</v>
-      </c>
-      <c r="X47" t="n">
-        <v>-0.31</v>
+        <v>-4.8</v>
       </c>
       <c r="Y47" t="n">
-        <v>10</v>
+        <v>-16.4</v>
       </c>
       <c r="Z47" t="n">
-        <v>482.147</v>
+        <v>1.795</v>
       </c>
       <c r="AA47" t="n">
-        <v>-25.78</v>
+        <v>-1.98</v>
       </c>
       <c r="AB47" t="n">
-        <v>15.9</v>
+        <v>-0</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>0.62</v>
       </c>
       <c r="AF47" t="inlineStr">
         <is>
@@ -3752,62 +3710,63 @@
       </c>
       <c r="AG47" t="inlineStr">
         <is>
-          <t>reports/saudi-arabia-sovereign-credit.md</t>
+          <t>reports/rwanda-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa (WAEMU)</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>CC</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>Caa2</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Staff-level agreement on new arrangement replacing suspended USD 1.8B facility; Board consideration 15-Dec-26</t>
-        </is>
-      </c>
+          <t>Middle East</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr"/>
       <c r="G48" t="n">
-        <v>6.8</v>
+        <v>3.1</v>
       </c>
       <c r="H48" t="n">
-        <v>1.2</v>
+        <v>1.82</v>
       </c>
       <c r="I48" t="n">
-        <v>3</v>
+        <v>4.5</v>
       </c>
       <c r="J48" t="n">
-        <v>1.8</v>
+        <v>2.68</v>
       </c>
       <c r="K48" t="n">
-        <v>-6.2</v>
+        <v>-1.6</v>
+      </c>
+      <c r="L48" t="n">
+        <v>488.684</v>
+      </c>
+      <c r="M48" t="n">
+        <v>15.6</v>
       </c>
       <c r="P48" t="n">
-        <v>132</v>
+        <v>32.1</v>
       </c>
       <c r="Q48" t="n">
-        <v>-6.7</v>
+        <v>-3.5</v>
+      </c>
+      <c r="X48" t="n">
+        <v>-0.31</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>10</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>482.147</v>
+      </c>
+      <c r="AA48" t="n">
+        <v>-25.78</v>
       </c>
       <c r="AB48" t="n">
-        <v>-2.4</v>
-      </c>
-      <c r="AC48" t="n">
-        <v>3.2</v>
+        <v>15.9</v>
       </c>
       <c r="AF48" t="inlineStr">
         <is>
@@ -3816,82 +3775,62 @@
       </c>
       <c r="AG48" t="inlineStr">
         <is>
-          <t>reports/senegal-sovereign-credit.md</t>
+          <t>reports/saudi-arabia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CEEMEA - Western Balkans</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>BB+</t>
+          <t>Sub-Saharan Africa (WAEMU)</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>BBB-</t>
+          <t>CC</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Ba2</t>
+          <t>Caa2</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Policy Coordination Instrument (36-month, non-financing)</t>
+          <t>Staff-level agreement on new arrangement replacing suspended USD 1.8B facility; Board consideration 15-Dec-26</t>
         </is>
       </c>
       <c r="G49" t="n">
-        <v>3.8</v>
+        <v>6.8</v>
       </c>
       <c r="H49" t="n">
-        <v>2.2</v>
+        <v>1.2</v>
       </c>
       <c r="I49" t="n">
-        <v>5.75</v>
+        <v>3</v>
       </c>
       <c r="J49" t="n">
-        <v>3.55</v>
+        <v>1.8</v>
       </c>
       <c r="K49" t="n">
-        <v>-4.1</v>
-      </c>
-      <c r="L49" t="n">
-        <v>35.71</v>
-      </c>
-      <c r="M49" t="n">
-        <v>6.2</v>
+        <v>-6.2</v>
       </c>
       <c r="P49" t="n">
-        <v>43.3</v>
+        <v>132</v>
       </c>
       <c r="Q49" t="n">
-        <v>-3.25</v>
-      </c>
-      <c r="X49" t="n">
-        <v>1.37</v>
-      </c>
-      <c r="Y49" t="n">
-        <v>7</v>
-      </c>
-      <c r="Z49" t="n">
-        <v>30.033</v>
-      </c>
-      <c r="AA49" t="n">
-        <v>-4.36</v>
+        <v>-6.7</v>
       </c>
       <c r="AB49" t="n">
-        <v>-1.4</v>
+        <v>-2.4</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>3.2</v>
       </c>
       <c r="AF49" t="inlineStr">
         <is>
@@ -3900,29 +3839,29 @@
       </c>
       <c r="AG49" t="inlineStr">
         <is>
-          <t>reports/serbia-sovereign-credit.md</t>
+          <t>reports/senegal-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>South Africa</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Sub-Saharan Africa</t>
+          <t>CEEMEA - Western Balkans</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BB+</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>BBB-</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -3932,53 +3871,50 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>None (Article IV)</t>
+          <t>Policy Coordination Instrument (36-month, non-financing)</t>
         </is>
       </c>
       <c r="G50" t="n">
-        <v>1</v>
+        <v>3.8</v>
       </c>
       <c r="H50" t="n">
-        <v>4.4</v>
+        <v>2.2</v>
       </c>
       <c r="I50" t="n">
-        <v>7.25</v>
+        <v>5.75</v>
       </c>
       <c r="J50" t="n">
-        <v>2.9</v>
+        <v>3.55</v>
       </c>
       <c r="K50" t="n">
-        <v>-1.6</v>
+        <v>-4.1</v>
       </c>
       <c r="L50" t="n">
-        <v>75.95999999999999</v>
+        <v>35.71</v>
       </c>
       <c r="M50" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
       <c r="P50" t="n">
-        <v>77.2</v>
+        <v>43.3</v>
       </c>
       <c r="Q50" t="n">
-        <v>-3.8</v>
-      </c>
-      <c r="S50" t="n">
-        <v>20</v>
+        <v>-3.25</v>
       </c>
       <c r="X50" t="n">
-        <v>1.23</v>
+        <v>1.37</v>
       </c>
       <c r="Y50" t="n">
-        <v>7.8</v>
+        <v>7</v>
       </c>
       <c r="Z50" t="n">
-        <v>74.307</v>
+        <v>30.033</v>
       </c>
       <c r="AA50" t="n">
-        <v>-1.32</v>
+        <v>-4.36</v>
       </c>
       <c r="AB50" t="n">
-        <v>-0.9</v>
+        <v>-1.4</v>
       </c>
       <c r="AF50" t="inlineStr">
         <is>
@@ -3987,51 +3923,85 @@
       </c>
       <c r="AG50" t="inlineStr">
         <is>
-          <t>reports/south-africa-sovereign-credit.md</t>
+          <t>reports/serbia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>South Africa</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Central Asia</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr"/>
+          <t>Sub-Saharan Africa</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>None (Article IV)</t>
+        </is>
+      </c>
       <c r="G51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="H51" t="n">
-        <v>4.0609</v>
+        <v>4.4</v>
+      </c>
+      <c r="I51" t="n">
+        <v>7.25</v>
+      </c>
+      <c r="J51" t="n">
+        <v>2.9</v>
       </c>
       <c r="K51" t="n">
-        <v>6.3</v>
+        <v>-1.6</v>
       </c>
       <c r="L51" t="n">
-        <v>6.395</v>
+        <v>75.95999999999999</v>
       </c>
       <c r="M51" t="n">
-        <v>5.749</v>
+        <v>5.8</v>
       </c>
       <c r="P51" t="n">
-        <v>21.9</v>
+        <v>77.2</v>
       </c>
       <c r="Q51" t="n">
-        <v>-2.5</v>
+        <v>-3.8</v>
+      </c>
+      <c r="S51" t="n">
+        <v>20</v>
+      </c>
+      <c r="X51" t="n">
+        <v>1.23</v>
       </c>
       <c r="Y51" t="n">
-        <v>45.9</v>
+        <v>7.8</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>74.307</v>
       </c>
       <c r="AA51" t="n">
-        <v>3.48</v>
+        <v>-1.32</v>
       </c>
       <c r="AB51" t="n">
-        <v>-0.8</v>
+        <v>-0.9</v>
       </c>
       <c r="AF51" t="inlineStr">
         <is>
@@ -4040,228 +4010,195 @@
       </c>
       <c r="AG51" t="inlineStr">
         <is>
-          <t>reports/tajikistan-sovereign-credit.md</t>
+          <t>reports/south-africa-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Asia</t>
+          <t>Central Asia</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="H52" t="n">
-        <v>2.5265</v>
-      </c>
-      <c r="I52" t="n">
-        <v>1</v>
-      </c>
-      <c r="J52" t="n">
-        <v>-1.53</v>
+        <v>4.0609</v>
       </c>
       <c r="K52" t="n">
-        <v>0.7</v>
+        <v>6.3</v>
       </c>
       <c r="L52" t="n">
-        <v>283.137</v>
+        <v>6.395</v>
       </c>
       <c r="M52" t="n">
-        <v>8.051</v>
+        <v>5.749</v>
       </c>
       <c r="P52" t="n">
-        <v>66.8</v>
+        <v>21.9</v>
       </c>
       <c r="Q52" t="n">
-        <v>-2.2</v>
-      </c>
-      <c r="X52" t="n">
-        <v>0.21</v>
+        <v>-2.5</v>
       </c>
       <c r="Y52" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="Z52" t="n">
-        <v>302.852</v>
+        <v>45.9</v>
       </c>
       <c r="AA52" t="n">
-        <v>8.08</v>
+        <v>3.48</v>
       </c>
       <c r="AB52" t="n">
-        <v>-3.9</v>
+        <v>-0.8</v>
       </c>
       <c r="AF52" t="inlineStr">
         <is>
-          <t>08-Oct-26</t>
+          <t>09-Oct-26</t>
         </is>
       </c>
       <c r="AG52" t="inlineStr">
         <is>
-          <t>reports/thailand-sovereign-credit.md</t>
+          <t>reports/tajikistan-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>North Africa</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>B-</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Caa1</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>$1.9bn Extended Fund Facility agreed at staff level Oct-22; never approved by the Executive Board; frozen</t>
-        </is>
-      </c>
+          <t>Asia</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr"/>
       <c r="G53" t="n">
-        <v>2.1</v>
+        <v>1.5</v>
       </c>
       <c r="H53" t="n">
-        <v>5.6</v>
+        <v>2.5265</v>
       </c>
       <c r="I53" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="J53" t="n">
-        <v>1.4</v>
+        <v>-1.53</v>
       </c>
       <c r="K53" t="n">
-        <v>-4.2</v>
+        <v>0.7</v>
       </c>
       <c r="L53" t="n">
-        <v>9.079000000000001</v>
+        <v>283.137</v>
       </c>
       <c r="M53" t="n">
-        <v>3</v>
+        <v>8.051</v>
       </c>
       <c r="P53" t="n">
-        <v>82</v>
+        <v>66.8</v>
       </c>
       <c r="Q53" t="n">
-        <v>-5.2</v>
+        <v>-2.2</v>
       </c>
       <c r="X53" t="n">
-        <v>1.63</v>
+        <v>0.21</v>
       </c>
       <c r="Y53" t="n">
-        <v>6.8</v>
+        <v>5.9</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>302.852</v>
       </c>
       <c r="AA53" t="n">
-        <v>-1.33</v>
+        <v>8.08</v>
       </c>
       <c r="AB53" t="n">
-        <v>-1.2</v>
-      </c>
-      <c r="AC53" t="n">
-        <v>0.15</v>
+        <v>-3.9</v>
       </c>
       <c r="AF53" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>08-Oct-26</t>
         </is>
       </c>
       <c r="AG53" t="inlineStr">
         <is>
-          <t>reports/tunisia-sovereign-credit.md</t>
+          <t>reports/thailand-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CEEMEA</t>
+          <t>North Africa</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BB-</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>BB-</t>
+          <t>B-</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Ba3</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr"/>
+          <t>Caa1</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>$1.9bn Extended Fund Facility agreed at staff level Oct-22; never approved by the Executive Board; frozen</t>
+        </is>
+      </c>
       <c r="G54" t="n">
-        <v>3.4</v>
+        <v>2.1</v>
       </c>
       <c r="H54" t="n">
-        <v>29.73</v>
+        <v>5.6</v>
       </c>
       <c r="I54" t="n">
-        <v>37</v>
+        <v>7</v>
       </c>
       <c r="J54" t="n">
-        <v>12.5</v>
+        <v>1.4</v>
       </c>
       <c r="K54" t="n">
-        <v>-2.7</v>
+        <v>-4.2</v>
       </c>
       <c r="L54" t="n">
-        <v>174.4</v>
+        <v>9.079000000000001</v>
       </c>
       <c r="M54" t="n">
-        <v>5.128</v>
-      </c>
-      <c r="N54" t="n">
-        <v>1.02</v>
-      </c>
-      <c r="O54" t="n">
-        <v>31.8</v>
+        <v>3</v>
       </c>
       <c r="P54" t="n">
-        <v>29.5</v>
+        <v>82</v>
       </c>
       <c r="Q54" t="n">
         <v>-5.2</v>
       </c>
       <c r="X54" t="n">
-        <v>0.31</v>
+        <v>1.63</v>
       </c>
       <c r="Y54" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="Z54" t="n">
-        <v>137.109</v>
+        <v>6.8</v>
       </c>
       <c r="AA54" t="n">
-        <v>-38.89</v>
+        <v>-1.33</v>
       </c>
       <c r="AB54" t="n">
-        <v>-1</v>
+        <v>-1.2</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>0.15</v>
       </c>
       <c r="AF54" t="inlineStr">
         <is>
@@ -4270,14 +4207,14 @@
       </c>
       <c r="AG54" t="inlineStr">
         <is>
-          <t>reports/turkey-sovereign-credit.md</t>
+          <t>reports/tunisia-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Ukraine</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4287,65 +4224,67 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>CCC+</t>
+          <t>BB-</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Ca</t>
-        </is>
-      </c>
-      <c r="F55" t="inlineStr">
-        <is>
-          <t>4-year EFF (first review completed 20-Jul-26, SDR 503M, about $690M disbursed)</t>
-        </is>
-      </c>
+          <t>Ba3</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>2</v>
+        <v>3.4</v>
       </c>
       <c r="H55" t="n">
-        <v>8.1</v>
+        <v>29.73</v>
       </c>
       <c r="I55" t="n">
-        <v>16</v>
+        <v>37</v>
       </c>
       <c r="J55" t="n">
-        <v>7.9</v>
+        <v>12.5</v>
       </c>
       <c r="K55" t="n">
-        <v>-18.9</v>
+        <v>-2.7</v>
       </c>
       <c r="L55" t="n">
-        <v>47.1</v>
+        <v>174.4</v>
       </c>
       <c r="M55" t="n">
-        <v>5.6</v>
+        <v>5.128</v>
+      </c>
+      <c r="N55" t="n">
+        <v>1.02</v>
+      </c>
+      <c r="O55" t="n">
+        <v>31.8</v>
       </c>
       <c r="P55" t="n">
-        <v>98.40000000000001</v>
+        <v>29.5</v>
       </c>
       <c r="Q55" t="n">
-        <v>-18.4</v>
+        <v>-5.2</v>
       </c>
       <c r="X55" t="n">
-        <v>-0.5</v>
+        <v>0.31</v>
       </c>
       <c r="Y55" t="n">
-        <v>5.7</v>
+        <v>4.7</v>
       </c>
       <c r="Z55" t="n">
-        <v>38.646</v>
+        <v>137.109</v>
       </c>
       <c r="AA55" t="n">
-        <v>-24.81</v>
+        <v>-38.89</v>
       </c>
       <c r="AB55" t="n">
-        <v>-2.3</v>
+        <v>-1</v>
       </c>
       <c r="AF55" t="inlineStr">
         <is>
@@ -4354,61 +4293,82 @@
       </c>
       <c r="AG55" t="inlineStr">
         <is>
-          <t>reports/ukraine-sovereign-credit.md</t>
+          <t>reports/turkey-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Ukraine</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MENA / GCC</t>
+          <t>CEEMEA</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>AA-</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>AA</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr"/>
+          <t>CCC+</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Ca</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>4-year EFF (first review completed 20-Jul-26, SDR 503M, about $690M disbursed)</t>
+        </is>
+      </c>
       <c r="G56" t="n">
-        <v>3.1</v>
+        <v>2</v>
       </c>
       <c r="H56" t="n">
-        <v>2.05</v>
+        <v>8.1</v>
+      </c>
+      <c r="I56" t="n">
+        <v>16</v>
+      </c>
+      <c r="J56" t="n">
+        <v>7.9</v>
       </c>
       <c r="K56" t="n">
-        <v>11.4</v>
+        <v>-18.9</v>
       </c>
       <c r="L56" t="n">
-        <v>259.7</v>
+        <v>47.1</v>
       </c>
       <c r="M56" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="P56" t="n">
-        <v>31.4</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="Q56" t="n">
-        <v>4.9</v>
+        <v>-18.4</v>
       </c>
       <c r="X56" t="n">
-        <v>-1.12</v>
+        <v>-0.5</v>
       </c>
       <c r="Y56" t="n">
-        <v>-3.1</v>
+        <v>5.7</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>38.646</v>
+      </c>
+      <c r="AA56" t="n">
+        <v>-24.81</v>
       </c>
       <c r="AB56" t="n">
-        <v>13.2</v>
+        <v>-2.3</v>
       </c>
       <c r="AF56" t="inlineStr">
         <is>
@@ -4417,73 +4377,61 @@
       </c>
       <c r="AG56" t="inlineStr">
         <is>
-          <t>reports/uae-sovereign-credit.md</t>
+          <t>reports/ukraine-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Uzbekistan</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Central Asia / CIS</t>
+          <t>MENA / GCC</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>BB</t>
+          <t>AA-</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>BB</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Ba2</t>
-        </is>
-      </c>
-      <c r="F57" t="inlineStr">
-        <is>
-          <t>None (Article IV surveillance only)</t>
-        </is>
-      </c>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr"/>
       <c r="G57" t="n">
-        <v>8.699999999999999</v>
+        <v>3.1</v>
       </c>
       <c r="H57" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="I57" t="n">
-        <v>14</v>
-      </c>
-      <c r="J57" t="n">
-        <v>7.8</v>
+        <v>2.05</v>
       </c>
       <c r="K57" t="n">
-        <v>-1.3</v>
+        <v>11.4</v>
       </c>
       <c r="L57" t="n">
-        <v>72.13</v>
+        <v>259.7</v>
       </c>
       <c r="M57" t="n">
-        <v>12</v>
+        <v>5.2</v>
       </c>
       <c r="P57" t="n">
-        <v>27</v>
+        <v>31.4</v>
       </c>
       <c r="Q57" t="n">
-        <v>-2.1</v>
+        <v>4.9</v>
+      </c>
+      <c r="X57" t="n">
+        <v>-1.12</v>
       </c>
       <c r="Y57" t="n">
-        <v>32</v>
-      </c>
-      <c r="AA57" t="n">
-        <v>-11.23</v>
+        <v>-3.1</v>
+      </c>
+      <c r="AB57" t="n">
+        <v>13.2</v>
       </c>
       <c r="AF57" t="inlineStr">
         <is>
@@ -4492,89 +4440,164 @@
       </c>
       <c r="AG57" t="inlineStr">
         <is>
-          <t>reports/uzbekistan-sovereign-credit.md</t>
+          <t>reports/uae-sovereign-credit.md</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>Uzbekistan</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Central Asia / CIS</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>BB</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Ba2</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>None (Article IV surveillance only)</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="H58" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="I58" t="n">
+        <v>14</v>
+      </c>
+      <c r="J58" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="K58" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="L58" t="n">
+        <v>72.13</v>
+      </c>
+      <c r="M58" t="n">
+        <v>12</v>
+      </c>
+      <c r="P58" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>-2.1</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>32</v>
+      </c>
+      <c r="AA58" t="n">
+        <v>-11.23</v>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>09-Oct-26</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>reports/uzbekistan-sovereign-credit.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>Zambia</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Sub-Saharan Africa</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>B-</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>CCC+</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Caa2</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>38-month ECF completed Jan-26 (sixth and final review); successor programme under negotiation</t>
         </is>
       </c>
-      <c r="G58" t="n">
+      <c r="G59" t="n">
         <v>4.3</v>
       </c>
-      <c r="H58" t="n">
+      <c r="H59" t="n">
         <v>6.1</v>
       </c>
-      <c r="I58" t="n">
+      <c r="I59" t="n">
         <v>10.75</v>
       </c>
-      <c r="J58" t="n">
+      <c r="J59" t="n">
         <v>4.65</v>
       </c>
-      <c r="K58" t="n">
+      <c r="K59" t="n">
         <v>0.9</v>
       </c>
-      <c r="L58" t="n">
+      <c r="L59" t="n">
         <v>5.8</v>
       </c>
-      <c r="M58" t="n">
+      <c r="M59" t="n">
         <v>4.2</v>
       </c>
-      <c r="P58" t="n">
+      <c r="P59" t="n">
         <v>91</v>
       </c>
-      <c r="Q58" t="n">
+      <c r="Q59" t="n">
         <v>-4.9</v>
       </c>
-      <c r="S58" t="n">
+      <c r="S59" t="n">
         <v>35</v>
       </c>
-      <c r="X58" t="n">
+      <c r="X59" t="n">
         <v>2.27</v>
       </c>
-      <c r="Y58" t="n">
+      <c r="Y59" t="n">
         <v>25.6</v>
       </c>
-      <c r="AA58" t="n">
+      <c r="AA59" t="n">
         <v>-0.9</v>
       </c>
-      <c r="AB58" t="n">
+      <c r="AB59" t="n">
         <v>5.1</v>
       </c>
-      <c r="AF58" t="inlineStr">
+      <c r="AF59" t="inlineStr">
         <is>
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="AG58" t="inlineStr">
+      <c r="AG59" t="inlineStr">
         <is>
           <t>reports/zambia-sovereign-credit.md</t>
         </is>

</xml_diff>

<commit_message>
site build 2026-10-19 08:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -4238,7 +4238,7 @@
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="n">
-        <v>3.4</v>
+        <v>2.8</v>
       </c>
       <c r="H55" t="n">
         <v>29.73</v>
@@ -4253,13 +4253,13 @@
         <v>-2.7</v>
       </c>
       <c r="L55" t="n">
-        <v>174.4</v>
+        <v>167.4</v>
       </c>
       <c r="M55" t="n">
         <v>5.128</v>
       </c>
       <c r="N55" t="n">
-        <v>1.02</v>
+        <v>0.98</v>
       </c>
       <c r="O55" t="n">
         <v>31.8</v>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="AF55" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>19-Oct-26</t>
         </is>
       </c>
       <c r="AG55" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-19 10:04
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -4324,7 +4324,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>4-year EFF (first review completed 20-Jul-26; SDR 503M, about $690M disbursed)</t>
+          <t>4-year EFF</t>
         </is>
       </c>
       <c r="G56" t="n">
@@ -4371,7 +4371,7 @@
       </c>
       <c r="AF56" t="inlineStr">
         <is>
-          <t>09-Oct-26</t>
+          <t>19-Oct-26</t>
         </is>
       </c>
       <c r="AG56" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-27 12:05
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -426,7 +426,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Sovereign comp sheet, built 26-Oct-26 from database/sovereigns/*.json; derived columns are formulas on the Data sheet</t>
+          <t>Sovereign comp sheet, built 27-Oct-26 from database/sovereigns/*.json; derived columns are formulas on the Data sheet</t>
         </is>
       </c>
     </row>
@@ -4247,22 +4247,22 @@
         <v>29.73</v>
       </c>
       <c r="I55" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J55" t="n">
-        <v>12.5</v>
+        <v>12.11</v>
       </c>
       <c r="K55" t="n">
         <v>-2.7</v>
       </c>
       <c r="L55" t="n">
-        <v>167.4</v>
+        <v>171.6</v>
       </c>
       <c r="M55" t="n">
         <v>5.128</v>
       </c>
       <c r="N55" t="n">
-        <v>0.98</v>
+        <v>1.01</v>
       </c>
       <c r="O55" t="n">
         <v>31.8</v>
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AF55" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>27-Oct-26</t>
         </is>
       </c>
       <c r="AG55" t="inlineStr">

</xml_diff>

<commit_message>
site build 2026-10-28 20:45
</commit_message>
<xml_diff>
--- a/models/sovereigns/Sovereign_Comp_Sheet.xlsx
+++ b/models/sovereigns/Sovereign_Comp_Sheet.xlsx
@@ -426,7 +426,7 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Sovereign comp sheet, built 27-Oct-26 from database/sovereigns/*.json; derived columns are formulas on the Data sheet</t>
+          <t>Sovereign comp sheet, built 28-Oct-26 from database/sovereigns/*.json; derived columns are formulas on the Data sheet</t>
         </is>
       </c>
     </row>
@@ -4334,13 +4334,13 @@
         <v>2</v>
       </c>
       <c r="H56" t="n">
-        <v>8.1</v>
+        <v>10</v>
       </c>
       <c r="I56" t="n">
         <v>16</v>
       </c>
       <c r="J56" t="n">
-        <v>7.9</v>
+        <v>6</v>
       </c>
       <c r="K56" t="n">
         <v>-18.9</v>
@@ -4374,7 +4374,7 @@
       </c>
       <c r="AF56" t="inlineStr">
         <is>
-          <t>19-Oct-26</t>
+          <t>28-Oct-26</t>
         </is>
       </c>
       <c r="AG56" t="inlineStr">

</xml_diff>